<commit_message>
[Excel] Add [FR] "annotation" column translation for OWASP Top 10 Web - 2025
</commit_message>
<xml_diff>
--- a/tools/excel/owasp/owasp-top-10-web_2025.xlsx
+++ b/tools/excel/owasp/owasp-top-10-web_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\owasp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3413A75-EE7C-4BF5-8441-D5798469F514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F5AF1F-7CFE-4CA5-8CC4-7BED21A95881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="387">
   <si>
     <t>type</t>
   </si>
@@ -7946,12 +7946,683 @@
 Un logiciel sécurisé nécessite un cycle de développement sécurisé, un modèle de conception sécurisé, une méthodologie pavée, une bibliothèque de composants sécurisée, des outils appropriés, une modélisation des menaces et des post-mortem d’incidents utilisés pour améliorer le processus. Contactez vos spécialistes de la sécurité au début d’un projet logiciel, tout au long du projet, et pour la maintenance logicielle continue. Envisagez d’utiliser le [Modèle de Maturité d’Assurance Logicielle OWASP (SAMM)](https://owaspsamm.org/) pour structurer vos efforts de développement logiciel sécurisé. 
 Souvent, l’autoresponsabilité des développeurs est sous-estimée. Favoriser une culture de conscience, de responsabilité et d’atténuation proactive des risques. Des échanges réguliers sur la sécurité (par exemple lors de séances de modélisation des menaces) peuvent générer un état d’esprit visant à inclure la sécurité dans toutes les décisions de conception importantes.</t>
   </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;40
+   &lt;/td&gt;
+   &lt;td&gt;20,15 % 
+   &lt;/td&gt;
+   &lt;td&gt;3,74 % 
+   &lt;/td&gt;
+   &lt;td&gt;100,00 % 
+   &lt;/td&gt;
+   &lt;td&gt;42,93 % 
+   &lt;/td&gt;
+   &lt;td&gt;7.04
+   &lt;/td&gt;
+   &lt;td&gt;3,84
+   &lt;/td&gt;
+   &lt;td&gt;1 839 701
+   &lt;/td&gt;
+   &lt;td&gt;32 654
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+Le contrôle d’accès n’est efficace que lorsqu’il est implémenté dans du code serveur de confiance ou dans des API serverless, où l’attaquant ne peut pas modifier la vérification ou les métadonnées de contrôle d’accès. 
+* Sauf pour les ressources publiques, refuser par défaut. 
+* Implémenter les mécanismes de contrôle d’accès une fois et les réutiliser dans toute l’application, y compris en minimisant l’utilisation du partage de ressources inter-origine (CORS). 
+* Les contrôles d’accès aux modèles devraient imposer la propriété des enregistrements plutôt que de permettre aux utilisateurs de créer, lire, mettre à jour ou supprimer un enregistrement. 
+* Les exigences uniques de limite d’activité des applications doivent être appliquées par les modèles de domaine. 
+* Désactivez la liste des répertoires des serveurs web et assurez-vous que les métadonnées de fichiers (par exemple, .git) et les fichiers de sauvegarde ne sont pas présents dans les racines web. 
+* Échecs de contrôle d’accès aux journaux, alerter les administrateurs lorsque cela est approprié (par exemple, échecs répétés). 
+* Mettre en place des limites de vitesse sur l’accès à l’API et aux contrôleurs afin de minimiser les dommages causés par les outils d’attaque automatisés. 
+* Les identifiants de session avec état doivent être invalidés sur le serveur après la déconnexion. Les jetons JWT sans état doivent être de courte durée afin de minimiser la fenêtre d’opportunité pour un attaquant. Pour les JWT à durée de vie plus longue, envisagez d’utiliser des jetons de rafraîchissement et de suivre les normes OAuth pour révoquer l’accès. 
+* Utilisez des kits à outils ou des motifs bien établis qui fournissent des contrôles d’accès simples et déclaratifs. 
+Les développeurs et le personnel QA devraient inclure le contrôle d’accès fonctionnel dans leurs tests unitaires et d’intégration.
+## Exemples de scénarios d’attaque
+**Scénario #1 :** L’application utilise des données non vérifiées dans un appel SQL qui accédent aux informations du compte : 
+```
+pstmt.setString(1, request.getParameter(« acct »)) ; 
+ResultSet results = pstmt.executeQuery( ) ; 
+```
+Un attaquant peut simplement modifier le paramètre « compte » du navigateur pour envoyer n’importe quel numéro de compte souhaité. Si ce n’est pas correctement vérifié, l’attaquant peut accéder au compte de n’importe quel utilisateur. 
+```
+https://example.com/app/accountInfo?acct=notmyacct
+```
+**Scénario #2 :** Un attaquant force simplement les navigateurs à cibler les URL. Des droits d’administrateur sont nécessaires pour accéder à la page d’administration. 
+```
+https://example.com/app/getappInfo
+https://example.com/app/admin_getappInfo
+```
+Si un utilisateur non authentifié peut accéder à l’une ou l’autre des pages, c’est un défaut. Si un non-administrateur peut accéder à la page d’administration, c’est un défaut. 
+**Scénario #3 :** Une application met tout son contrôle d’accès dans son front-end. Bien que l’attaquant ne puisse pas accéder à « https://example.com/app/admin_getappInfo » en raison du code JavaScript qui tourne dans le navigateur, il peut simplement exécuter : 
+```
+$ curl https://example.com/app/admin_getappInfo
+```
+depuis la ligne de commande. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A01_2025-Broken_Access_Control/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;16
+   &lt;/td&gt;
+   &lt;td&gt;27,70 % 
+   &lt;/td&gt;
+   &lt;td&gt;3,00 % 
+   &lt;/td&gt;
+   &lt;td&gt;100,00 % 
+   &lt;/td&gt;
+   &lt;td&gt;52,35 % 
+   &lt;/td&gt;
+   &lt;td&gt;7,96
+   &lt;/td&gt;
+   &lt;td&gt;3,97
+   &lt;/td&gt;
+   &lt;td&gt;719 084
+   &lt;/td&gt;
+   &lt;td&gt;1 375
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+Des processus d’installation sécurisés doivent être mis en œuvre, notamment : 
+* Un processus de durcissement répétable permettant un déploiement rapide et facile d’un autre environnement suffisamment verrouillé. Les environnements de développement, d’assurance qualité et de production doivent tous être configurés de manière identique, avec des identifiants différents utilisés dans chaque environnement. Ce processus doit être automatisé pour minimiser l’effort nécessaire à la mise en place d’un nouvel environnement sécurisé. 
+* Une plateforme minimale sans fonctionnalités, composants, documentations ou exemples inutiles. Supprimez ou n’installez pas les fonctionnalités et frameworks inutilisés. 
+* Une tâche visant à revoir et mettre à jour les configurations appropriées à toutes les notes de sécurité, mises à jour et correctifs dans le cadre du processus de gestion des correctifs (voir [A03 Défaillances de la chaîne d’approvisionnement logicielle](A03_2025-Software_Supply_Chain_Failures.md)). Revoir les permissions de stockage cloud (par exemple, les permissions de bucket S3). 
+* Une architecture d’application segmentée offre une séparation efficace et sécurisée entre composants ou locataires, avec segmentation, conteneurisation ou groupes de sécurité cloud (ACL). 
+* Envoi de directives de sécurité aux clients, par exemple, les en-têtes de sécurité. 
+* Un processus automatisé pour vérifier l’efficacité des configurations et des réglages dans tous les environnements. 
+* Ajouter proactivement une configuration centrale pour intercepter les messages d’erreur excessifs en tant que sauvegarde. 
+* Si ces vérifications ne sont pas automatisées, elles doivent être vérifiées manuellement au minimum chaque année. 
+* Utiliser la fédération d’identité, des identifiants de courte durée ou des mécanismes d’accès basés sur des rôles fournis par la plateforme sous-jacente au lieu d’intégrer des clés statiques ou des secrets dans le code, les fichiers de configuration ou les pipelines.
+## Exemples de scénarios d’attaque
+**Scénario #1 :** Le serveur d’applications d’applications d’exemple n’est pas supprimé du serveur de production. Ces applications d’exemple présentent des failles de sécurité connues que les attaquants utilisent pour compromettre le serveur. Supposons que l’une de ces applications soit la console d’administration, et que les comptes par défaut n’aient pas été modifiés. Dans ce cas, l’attaquant se connecte avec le mot de passe par défaut et prend le relais. 
+**Scénario #2 :** La liste des répertoires n’est pas désactivée sur le serveur. Un attaquant découvre qu’il peut simplement lister les répertoires. L’attaquant trouve et télécharge les classes Java compilées, qu’il décompile et rétro-ingénierie pour visualiser le code. L’attaquant découvre alors une grave faille de contrôle d’accès dans l’application. 
+**Scénario #3 :** La configuration du serveur d’applications permet de renvoyer des messages d’erreur détaillés, tels que des traces de pile. Cela expose potentiellement des informations sensibles ou des failles sous-jacentes, comme des versions de composants connues pour être vulnérables. 
+**Scénario #4 :** Un fournisseur de services cloud (CSP) a par défaut des permissions de partage ouvertes à Internet. Cela permet d’accéder aux données sensibles stockées dans le stockage cloud. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A02_2025-Security_Misconfiguration/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;32
+   &lt;/td&gt;
+   &lt;td&gt;13,77 % 
+   &lt;/td&gt;
+   &lt;td&gt;3,80 % 
+   &lt;/td&gt;
+   &lt;td&gt;100,00 % 
+   &lt;/td&gt;
+   &lt;td&gt;47,74 % 
+   &lt;/td&gt;
+   &lt;td&gt;7.23
+   &lt;/td&gt;
+   &lt;td&gt;3,90
+   &lt;/td&gt;
+   &lt;td&gt;1 665 348
+   &lt;/td&gt;
+   &lt;td&gt;2 185
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+Faites au minimum ce qui suit et consultez les références : 
+* Classifier et étiqueter les données traitées, stockées ou transmises par une application. Identifier quelles données sont sensibles selon les lois sur la vie privée, les exigences réglementaires ou les besoins de l’entreprise. 
+* Stockez vos clés les plus sensibles dans un HSM matériel ou cloud. 
+* Utiliser des implémentations d’algorithmes cryptographiques bien fiables dans la mesure du possible. 
+* Ne stockez pas inutilement les données sensibles. Jetez-les dès que possible ou utilisez une tokenisation conforme PCI DSS, voire une troncature. Les données non conservées ne peuvent pas être volées. 
+* Assurez-vous de chiffrer toutes les données sensibles au repos. 
+* S’assurer que des algorithmes, protocoles et clés standards à jour et solides sont en place ; utiliser une gestion de clés appropriée. 
+* Chiffrer toutes les données en transit avec des protocoles &gt;= TLS 1.2 uniquement, avec des chiffrements de secret direct (FS), supprimer le support des chiffrements en chaîne de blocs de chiffrement (CBC), supporter les algorithmes de changement de clé quantique. Pour HTTPS, appliquer le chiffrement en utilisant HTTP Strict Transport Security (HSTS). Tout vérifier avec un outil. 
+* Désactivez la mise en cache pour les réponses contenant des données sensibles. Cela inclut la mise en cache dans votre CDN, votre serveur web et toute mise en cache d’application (par exemple : Redis). 
+* Appliquer les contrôles de sécurité requis selon la classification des données. 
+* N’utilisez pas de protocoles non chiffrés tels que FTP et STARTTLS. Évitez d’utiliser SMTP pour transmettre des données confidentielles. 
+* Stockez les mots de passe à l’aide de fonctions de hachage adaptatives fortes et salées avec un facteur de travail (facteur de retard), telles qu’Argon2, yescrypt, scrypt ou PBKDF2-HMAC-SHA-512. Pour les systèmes hérités utilisant bcrypt, obtenez plus de conseils sur [OWASP Cheat Sheet : Password Storage](https://cheatsheetseries.owasp.org/cheatsheets/Password_Storage_Cheat_Sheet.html)
+* Les vecteurs d’initialisation doivent être choisis en fonction du mode de fonctionnement. Cela peut signifier utiliser un CSPRNG (générateur de nombres pseudo aléatoires cryptographiquement sécurisé). Pour les modes nécessitant un nonce, le vecteur d’initialisation (IV) n’a pas besoin de CSPRNG. Dans tous les cas, l’IV ne doit jamais être utilisé deux fois pour une clé fixe. 
+* Utilisez toujours un chiffrement authentifié au lieu de simplement le chiffrement.
+* Les clés doivent être générées de manière cryptographique aléatoire et stockées en mémoire sous forme de tableaux d’octets. Si un mot de passe est utilisé, il doit alors être converti en clé via une fonction de dérivation de clé de base appropriée. 
+* S’assurer que l’aléa cryptographique est utilisée lorsque cela est approprié et qu’elle n’a pas été ensemencée de manière prévisible ou avec une faible entropie. La plupart des API modernes n’exigent pas que le développeur ensemence le CSPRNG pour être sécurisé. 
+* Éviter les fonctions cryptographiques obsolètes, les méthodes de construction de blocs et les schémas de remplissage, tels que MD5, SHA1, Cipher Block Chaining Mode (CBC), PKCS numéro 1 v1.5. 
+* Assurez-vous que les paramètres et configurations respectent les exigences de sécurité en les faisant examiner par des spécialistes de la sécurité, des outils conçus à cet effet, ou les deux. 
+* Vous devez vous préparer dès maintenant à la cryptographie post-quantique (PQC), voir référence (ENISA) afin que les systèmes à haut risque soient sûrs au plus tard fin 2030.
+## Exemples de scénarios d’attaque
+**Scénario #1** : Un site n’utilise pas et n’applique pas le TLS pour toutes les pages et ne supporte pas un chiffrement faible. Un attaquant surveille le trafic réseau (par exemple, sur un réseau sans fil non sécurisé), rétrograde les connexions de HTTPS à HTTP, intercepte les requêtes et vole le cookie de session de l’utilisateur. L’attaquant rejoue ensuite ce cookie et détourne la session (authentifiée) de l’utilisateur, accédant ou modifiant les données privées de l’utilisateur. Au lieu de ce qui précède, il pourrait modifier toutes les données transportées, par exemple le destinataire d’un transfert d’argent. 
+**Scénario #2** : La base de données de mots de passe utilise des hachages non salés ou simples pour stocker les mots de passe de chacun. Une faille de téléchargement de fichier permet à un attaquant de récupérer la base de mots de passe. Tous les hachages non salés peuvent être exposés avec une table arc-en-ciel de hachages pré-calculés. Les hachages générés par des fonctions de hachage simples ou rapides peuvent être cassés par des GPU, même s’ils ont été salés. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A04_2025-Cryptographic_Failures/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;37
+   &lt;/td&gt;
+   &lt;td&gt;13,77 % 
+   &lt;/td&gt;
+   &lt;td&gt;3,08 % 
+   &lt;/td&gt;
+   &lt;td&gt;100,00 % 
+   &lt;/td&gt;
+   &lt;td&gt;42,93 % 
+   &lt;/td&gt;
+   &lt;td&gt;7.15
+   &lt;/td&gt;
+   &lt;td&gt;4.32
+   &lt;/td&gt;
+   &lt;td&gt;1 404 249
+   &lt;/td&gt;
+   &lt;td&gt;62 445
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+Le meilleur moyen d’éviter l’injection consiste à séparer les données des commandes et requêtes : 
+* L’option préférée est d’utiliser une API sécurisée, qui évite complètement d’utiliser l’interpréteur, fournit une interface paramétrée ou migre vers des outils de cartographie relationnelle d’objets (ORM).  
+**Note :** Même paramétrés, les procédures stockées peuvent encore introduire l’injection SQL si PL/SQL ou T-SQL concaténe requêtes et données ou exécute des données hostiles avec EXECUTE IMMEDIATE ou exec(). 
+Lorsqu’il n’est pas possible de séparer les données des commandes, vous pouvez réduire les menaces en utilisant les techniques suivantes.  
+* Utilisez une validation d’entrée positive côté serveur. Ce n’est pas une défense complète car de nombreuses applications nécessitent des caractères spéciaux, tels que des zones de texte ou des API pour les applications mobiles. 
+* Pour toute requête dynamique résiduelle, échappez les caractères spéciaux en utilisant la syntaxe d’échappement spécifique de cet interpréteur.  
+**Note :** Les structures SQL telles que les noms de tables, les noms de colonnes, etc., ne peuvent pas être contournées, et donc les noms de structures fournis par l’utilisateur sont dangereux. C’est un problème courant dans les logiciels de rédaction de rapports. 
+**Attention** ces techniques impliquent l’analyse et l’évacuation de chaînes complexes, les rendant sujettes à l’erreur et peu robustes face à de légers changements du système sous-jacent.
+## Exemples de scénarios d’attaque
+**Scénario #1 :** Une application utilise des données non fiables dans la construction de l’appel SQL vulnérable suivant : 
+```
+Requête de chaîne = « SELECT * FROM accounts WHERE custID=' » + request.getParameter(« id ») + « ' » ; 
+```
+Un attaquant modifie la valeur du paramètre 'id' dans son navigateur pour envoyer : '' OU '1'='1'. Par exemple : 
+```
+http://example.com/app/accountView?id=' OU '1'='1
+```
+Cela modifie la signification de la requête pour retourner tous les enregistrements de la table des comptes. Des attaques plus dangereuses pourraient modifier ou supprimer des données, voire invoquer des procédures stockées. 
+**Scénario #2 :** La confiance aveugle d’une application dans les frameworks peut entraîner des requêtes qui restent vulnérables. Par exemple, Hibernate Query Language (HQL) : 
+```
+Requête HQLQuery = session.createQuery(« FROM accounts WHERE custID=' » + request.getParameter(« id ») + « ' ») ; 
+```
+Un attaquant fournit : « OR custID N’EST PAS NULL ni custID = ''. Cela contourne le filtre et renvoie tous les comptes. Bien que HQL ait moins de fonctions dangereuses que SQL brut, il permet toujours un accès non autorisé aux données lorsque les saisies de l’utilisateur sont concaténées en requêtes. 
+**Scénario #3 :** Une application transmet directement l’entrée utilisateur à une commande du système d’exploitation : 
+```
+String cmd = « nslookup " + request.getParameter(« domain ») ; 
+Runtime.getRuntime().exec(cmd) ; 
+```
+Un attaquant fournit des commandes arbitraires de type « example.com ; cat /etc/passwd » pour exécuter des commandes arbitraires sur le serveur. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A05_2025-Injection/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;36
+   &lt;/td&gt;
+   &lt;td&gt;15,80 % 
+   &lt;/td&gt;
+   &lt;td&gt;2,92 % 
+   &lt;/td&gt;
+   &lt;td&gt;100,00 % 
+   &lt;/td&gt;
+   &lt;td&gt;37,14 % 
+   &lt;/td&gt;
+   &lt;td&gt;7,69
+   &lt;/td&gt;
+   &lt;td&gt;4,44
+   &lt;/td&gt;
+   &lt;td&gt;1 120 673
+   &lt;/td&gt;
+   &lt;td&gt;7 147
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+* Lorsque possible, implémenter et faire respecter l’utilisation de l’authentification multifactorielle pour prévenir le bourrage automatisé des identifiants, la force brute et les attaques de réutilisation de crédents volées. 
+* Lorsque possible, encourager et activer l’utilisation de gestionnaires de mots de passe pour aider les utilisateurs à faire de meilleurs choix. 
+* Ne pas livrer ni déployer avec des identifiants par défaut, en particulier pour les utilisateurs administrateurs. 
+* Mettre en place des vérifications de mots de passe faibles, comme tester de nouveaux mots de passe ou modifiés dans la liste des 10 000 pires mots de passe. 
+* Lors de la création d’un nouveau compte et des changements de mot de passe, validez contre les listes d’identifiants connus pour violation (par exemple : utiliser [haveibeenpwned.com](https://haveibeenpwned.com)). 
+* Aligner les politiques de longueur, de complexité et de rotation des mots de passe avec les directives du [National Institute of Standards and Technology (NIST) 800-63b dans la section 5.1.1] (https://pages.nist.gov/800-63-3/sp800-63b.html#:~:text=5.1.1%20Memorized%20Secrets) pour les secrets mémorisés ou d’autres politiques modernes fondées sur des mots de passe fondées sur des preuves. 
+* Ne forcez pas les êtres humains à faire tourner les mots de passe sauf si vous suspectez une faille. Si vous soupçonnez une fuite, forcez immédiatement la réinitialisation du mot de passe.  
+* S’assurer que l’enregistrement, la récupération des identifiants et les voies API sont renforcés contre les attaques d’énumération de comptes en utilisant les mêmes messages pour tous les résultats (« Nom d’utilisateur ou mot de passe invalides. »). 
+* Limiter ou retarder de plus en plus les tentatives de connexion ratées, mais veillez à ne pas créer un scénario de déni de service. Consignez toutes les défaillances et alertez les administrateurs lorsque des attaques de type « credentialsal stuffing, de force brute » ou d’autres attaques sont détectées ou suspectées. 
+* Utiliser un gestionnaire de session intégré sécurisé côté serveur qui génère un nouvel ID de session aléatoire avec une forte entropie après la connexion. Les identifiants de session ne doivent pas être dans l’URL, être stockés de manière sécurisée dans un cookie sécurisé, et invalidés après déconnexion, inactivité et délais absolus.  
+* Idéalement, utiliser un système préfabriqué et bien fiable pour gérer l’authentification, l’identité et la gestion des sessions. Transférez ce risque autant que possible en achetant et en utilisant un système renforcé et bien testé. 
+* Vérifier l’utilisation prévue des identifiants fournis, par exemple pour les JWT, valider les affirmations « aud », « iss » et les périmètres
+## Exemples de scénarios d’attaque
+**Scénario #1 :** Le remplissage de crédentiaux, l’utilisation de listes de combinaisons de noms d’utilisateur et de mots de passe connus, est désormais une attaque très courante. Plus récemment, les attaquants ont été observés « incrémentant » ou ajustant autrement les mots de passe, en fonction du comportement humain courant. Par exemple, changer « Winter2025 » en « Hiver 2026 », ou « ILoveMyDog6 » en « ILoveMyDog7 » ou « ILoveMyDog5 ». Cet ajustement des tentatives de mot de passe est appelé attaque hybride de remplissage de crédibles ou attaque par pulvérisation de mots de passe, et ils peuvent être encore plus efficaces que la version traditionnelle. Si une application ne met pas en place de défenses contre les menaces automatisées (force brute, scripts ou bots) ou bourrage de crédents, l’application peut être utilisée comme oracle de mot de passe pour déterminer si les identifiants sont valides et obtenir un accès non autorisé. 
+**Scénario #2 :** La plupart des attaques d’authentification réussies surviennent en raison de l’utilisation continue des mots de passe comme seul facteur d’authentification. Une fois considérées comme les meilleures pratiques, la rotation des mots de passe et les exigences de complexité encouragent les utilisateurs à réutiliser les mots de passe et à utiliser des mots de passe faibles. Il est recommandé aux organisations d’arrêter ces pratiques conformément au NIST 800-63 et d’imposer l’utilisation de l’authentification multifacteur sur tous les systèmes importants. 
+**Scénario #3 :** Les délais d’expiration des sessions d’application ne sont pas correctement implémentés. Un utilisateur utilise un ordinateur public pour accéder à une application et au lieu de sélectionner « déconnexion », il ferme simplement l’onglet du navigateur et s’en va. Un autre exemple est si une session de connexion unique (SSO) ne peut pas être fermée par un seul déconnexion (SLO). C’est-à-dire qu’une seule connexion vous connecte, par exemple, à votre lecteur de messagerie, à votre système de documents et à votre système de chat. Mais la déconnexion ne se produit qu’au système actuel. Si un attaquant utilise le même navigateur après que la victime pense s’être déconnectée avec succès, mais avec l’utilisateur toujours authentifié sur certaines applications, il peut alors accéder au compte de la victime. Le même problème peut survenir dans les bureaux et les entreprises lorsqu’une application sensible n’a pas été correctement fermée et qu’un collègue a un accès (temporaire) à l’ordinateur déverrouillé. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A07_2025-Authentication_Failures/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;14
+   &lt;/td&gt;
+   &lt;td&gt;8,98 % 
+   &lt;/td&gt;
+   &lt;td&gt;2,75 % 
+   &lt;/td&gt;
+   &lt;td&gt;78,52 % 
+   &lt;/td&gt;
+   &lt;td&gt;45,49 % 
+   &lt;/td&gt;
+   &lt;td&gt;7.11
+   &lt;/td&gt;
+   &lt;td&gt;4,79
+   &lt;/td&gt;
+   &lt;td&gt;501 327
+   &lt;/td&gt;
+   &lt;td&gt;3 331
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+* Utilisez des signatures numériques ou des mécanismes similaires pour vérifier que le logiciel ou les données proviennent de la source attendue et n’ont pas été modifiés. 
+* Assurez-vous que les bibliothèques et dépendances, telles que npm ou Maven, ne consomment que des dépôts fiables. Si votre profil de risque est plus élevé, envisagez d’héberger un dépôt interne de bien connu qui est vérifié. 
+* Assurez-vous qu’un processus de révision des modifications de code et de configuration est en place afin de minimiser le risque que du code ou une configuration malveillante soit introduit dans votre pipeline logiciel. 
+* Assurez-vous que votre pipeline CI/CD dispose d’une ségrégation, d’une configuration et d’un contrôle d’accès appropriés afin d’assurer l’intégrité du code circulant dans les processus de compilation et de déploiement. 
+* S’assurer que les données sérialisées non signées ou non chiffrées ne sont pas reçues de clients non fiables et utilisées par la suite sans aucune forme de vérification d’intégrité ou de signature numérique pour détecter toute falsification ou relecture des données sérialisées.
+## Exemples de scénarios d’attaque
+**Scénario #1 Inclusion de fonctionnalités Web provenant d’une source non fiable :** Une entreprise utilise un fournisseur de services externe pour fournir des fonctionnalités de support. Pour plus de commodité, elle dispose d’une correspondance DNS pour « myCompany.SupportProvider.com » vers « support.myCompany.com ». Cela signifie que tous les cookies, y compris ceux d’authentification, définis sur le domaine « myCompany.com » seront désormais envoyés au fournisseur de support. Toute personne ayant accès à l’infrastructure du fournisseur de support peut voler les cookies de tous vos utilisateurs ayant visité « support.myCompany.com » et effectuer une attaque de détournement de session. 
+**Scénario #2 Mise à jour sans signature :** De nombreux routeurs domestiques, décodeurs, firmwares d’appareils et autres ne vérifient pas les mises à jour via un firmware signé. Le firmware non signé est une cible croissante pour les attaquants et devrait ne faire qu’empirer. C’est une préoccupation majeure car il n’existe souvent aucun mécanisme à remédier autre que de corriger dans une version future et d’attendre que les versions précédentes se dépassent. 
+**Scénario #3 Utilisation d’un paquet à partir d’une source non fiable :** Un développeur a du mal à trouver la version mise à jour d’un paquet qu’il recherche, il la télécharge donc non pas depuis le gestionnaire de paquets fiable classique, mais depuis un site web en ligne. Le paquet n’est pas signé, et il n’y a donc aucune possibilité d’en garantir l’intégrité. Le paquet inclut du code malveillant. 
+**Scénario #4 Désérialisation insécurisée :** Une application React appelle un ensemble de microservices Spring Boot. En tant que programmeurs fonctionnels, ils ont essayé de s’assurer que leur code reste immuable. La solution qu’ils ont trouvée est de sérialiser l’état utilisateur et de le transmettre à chaque requête. Un attaquant remarque la signature d’objet Java « rO0 » (en base64) et utilise le [Java Deserialization Scanner](https://github.com/federicodotta/Java-Deserialization-Scanner) pour obtenir une exécution de code à distance sur le serveur d’applications. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A08_2025-Software_or_Data_Integrity_Failures/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;24
+   &lt;/td&gt;
+   &lt;td&gt;20,67 % 
+   &lt;/td&gt;
+   &lt;td&gt;2,95 % 
+   &lt;/td&gt;
+   &lt;td&gt;100,00 % 
+   &lt;/td&gt;
+   &lt;td&gt;37,95 % 
+   &lt;/td&gt;
+   &lt;td&gt;7.11
+   &lt;/td&gt;
+   &lt;td&gt;3.81
+   &lt;/td&gt;
+   &lt;td&gt;769 581
+   &lt;/td&gt;
+   &lt;td&gt;3 416
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+Pour gérer correctement une condition exceptionnelle, nous devons planifier de telles situations (attendez-vous au pire). Nous devons « détecter » chaque erreur système possible directement à l’endroit où elle survient puis la traiter (ce qui signifie faire quelque chose de significatif pour résoudre le problème et nous assurer de nous en remettre). Dans le cadre de la gestion, nous devrions inclure l’envoi d’une erreur (pour informer l’utilisateur de manière compréhensible), la consignation de l’événement, ainsi que l’émission d’une alerte si cela est justifié. Nous devrions également avoir un gestionnaire global d’exceptions en place au cas où quelque chose serait manqué. Idéalement, nous aurions aussi des outils ou fonctionnalités de surveillance et/ou d’observabilité qui surveillent les erreurs répétées ou les schémas indiquant une attaque en cours, qui pourrait fournir une réponse, une défense ou un blocage quelconque. Cela peut nous aider à bloquer et à répondre aux scripts et bots qui se concentrent sur nos faiblesses en gestion des erreurs. 
+Détecter et gérer des conditions exceptionnelles garantit que l’infrastructure sous-jacente de nos programmes ne doit pas gérer des situations imprévisibles. Si vous êtes en cours de transaction de quelque nature que ce soit, il est extrêmement important de revenir en arrière sur chaque partie de la transaction et de recommencer (ce qu’on appelle également échec de clôture). Tenter de récupérer une transaction en cours de route est souvent l’occasion de créer des erreurs irrémédiables. 
+Dans la mesure du possible, ajoutez des limites de vitesse, des quotas de ressources, des limitations de puissance et d’autres limites autant que possible, pour prévenir des conditions exceptionnelles dès le départ. Rien dans les technologies de l’information ne devrait être illimité, car cela conduit à un manque de résilience des applications, au déni de service, à des attaques par force brute réussies et à des factures cloud extraordinaires. 
+Considérez si des erreurs répétées identiques, au-delà d’un certain débit, ne doivent être produites que sous forme de statistiques montrant la fréquence et dans quel délai ils se sont produits. Ces informations doivent être ajoutées au message original afin de ne pas interférer avec la journalisation et la surveillance automatisées, voir [A09:2025 Défaillances de journalisation et alertes de sécurité](A09_2025-Security_Logging_and_Alerting_Failures.md).
+En plus de cela, nous voudrions inclure une validation stricte des entrées (avec nettoyage ou échappement pour les caractères potentiellement dangereux que nous devons accepter), une gestion centralisée des erreurs, la journalisation, la surveillance et l’alerte, ainsi qu’un gestionnaire global d’exceptions. Une application ne doit pas avoir plusieurs fonctions pour gérer des conditions exceptionnelles, elle doit être effectuée en un seul endroit, de la même manière à chaque fois. Nous devrions également créer des exigences de sécurité du projet pour tous les conseils de cette section, effectuer la modélisation des menaces et/ou des activités de revue de conception sécurisée lors de la phase de conception de nos projets, effectuer des revues de code ou des analyses statiques, ainsi que réaliser des tests de stress, de performance et d’intrusion du système final. 
+Si possible, toute votre organisation devrait gérer les conditions exceptionnelles de la même manière, car cela facilite la relecture et l’audit du code pour détecter des erreurs dans ce contrôle de sécurité important.
+## Exemples de scénarios d’attaque
+**Scénario #1 : Une épuisement des ressources dû à une mauvaise gestion de conditions exceptionnelles (déni de service) peut être causé si l’application détecte des exceptions lors du téléchargement des fichiers, mais ne libère pas correctement les ressources ensuite. Chaque nouvelle exception laisse les ressources bloquées ou indisponibles, jusqu’à ce que toutes les ressources soient épuisées. 
+**Scénario #2 :** Exposition de données sensibles via une mauvaise gestion ou des erreurs de base de données qui révèlent l’erreur système complète à l’utilisateur. L’attaquant continue de forcer des erreurs afin d’utiliser les informations sensibles du système pour créer une meilleure attaque d’injection SQL. Les données sensibles dans les messages d’erreur utilisateur sont de la reconnaissance. 
+**Scénario #3 :** La corruption d’état dans les transactions financières pourrait être causée par un attaquant interrompant une transaction en plusieurs étapes via des perturbations réseau. Imaginez que l’ordre de la transaction soit : débiter un compte utilisateur, créditer le compte de destination, enregistrer la transaction. Si le système ne revient pas correctement sur l’intégralité de la transaction (échec fermé) en cas d’erreur en cours de route, l’attaquant pourrait potentiellement vider le compte de l’utilisateur, ou peut-être une condition de course permettant à l’attaquant d’envoyer de l’argent à destination plusieurs fois. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A10_2025-Mishandling_of_Exceptional_Conditions/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;6
+   &lt;/td&gt;
+   &lt;td&gt;9,56 % 
+   &lt;/td&gt;
+   &lt;td&gt;5,72 % 
+   &lt;/td&gt;
+   &lt;td&gt;65,42 % 
+   &lt;/td&gt;
+   &lt;td&gt;27,47 % 
+   &lt;/td&gt;
+   &lt;td&gt;8.17
+   &lt;/td&gt;
+   &lt;td&gt;5.23
+   &lt;/td&gt;
+   &lt;td&gt;215 248
+   &lt;/td&gt;
+   &lt;td&gt;11
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+Il devrait y avoir un processus de gestion des correctifs pour : 
+* Générer et gérer centralisément la liste des documents logiciels (SBOM) de l’ensemble de votre logiciel. 
+* Suivre non seulement vos dépendances directes, mais aussi leurs dépendances (transitives), et ainsi de suite. 
+* Réduire la surface d’attaque en supprimant les dépendances inutilisées, les fonctionnalités, les composants, les fichiers et la documentation inutiles. 
+* Inventorier continuellement les versions des composants côté client et côté serveur (par exemple, frameworks, bibliothèques) et leurs dépendances à l’aide d’outils comme OWASP Dependency Track, OWASP Dependency Check, retire.js, etc. 
+* Surveillez en continu des sources telles que Common Vulnerability and Exposures (CVE), National Vulnerability Database (NVD) et [Open Source Vulnerabilities (OSV)](https://osv.dev/) pour les vulnérabilités des composants que vous utilisez. Utilisez l’analyse de composition logicielle, la chaîne d’approvisionnement logicielle ou des outils SBOM axés sur la sécurité pour automatiser le processus. Abonnez-vous aux alertes concernant les vulnérabilités de sécurité liées aux composants que vous utilisez. 
+* N’obtenir les composants que de sources officielles (fiables) via des liens sécurisés. Privilégier les paquets signés pour réduire le risque d’inclure un composant modifié et malveillant (voir [A08:2025 - Défaillances d’intégrité logicielle et des données](https://owasp.org/Top10/2025/A08_2025-Software_or_Data_Integrity_Failures/)). 
+* Choisissez délibérément la version d’une dépendance que vous utilisez et ne mettez à jour que lorsqu’il y a un besoin. 
+* Surveillez les bibliothèques et composants non maintenus ou qui ne créent pas de correctifs de sécurité pour les versions précédentes. Si le patch n’est pas possible, envisagez de migrer vers une alternative. Si cela n’est pas possible, envisagez de déployer un correctif virtuel pour surveiller, détecter ou protéger contre le problème découvert. 
+* Mettez régulièrement à jour votre CI/CD, IDE et tout autre outil de développement
+* Éviter de déployer des mises à jour simultanément sur tous les systèmes. Utiliser des déploiements par étapes ou des déploiements canari pour limiter l’exposition au cas où un fournisseur de confiance serait compromis. 
+Il devrait y avoir un processus de gestion des changements ou un système de suivi pour suivre les modifications sur :
+* Paramètres CI/CD (tous les outils de compilation et pipelines)
+* Dépôts de code
+* Zones de bac à sable
+* IDE développeurs
+* Outils SBOM et artefacts créés
+* Systèmes de journalisation et journaux
+* Intégrations tierces, telles que le SaaS
+* Dépôts d’artefacts
+* Registres de conteneurs
+Renforcez les systèmes suivants, ce qui inclut la mise en service de la MFA et la fermeture de l’IAM : 
+* Votre dépôt de code (ce qui inclut de ne pas vérifier les secrets, protéger les branches, sauvegarder)
+* Stations de travail développeurs (correctifs réguliers, MFA, surveillance, et plus encore)
+* Votre serveur de compilation &amp; CI/CD (séparation des fonctions, contrôle d’accès, compilations signées, secrets à portée d’environnement, journaux inviolables, plus encore)
+* Vos artefacts (assurez l’intégrité via la provenance, la signature et l’horodatage, promouvez les artefacts plutôt que les reconstruisez pour chaque environnement, assurez-vous que les builds restent immuables)
+* Infrastructure en tant que code (géré comme tout le code, y compris l’utilisation des PR et le contrôle de versions)
+Chaque organisation doit s’assurer d’un plan continu pour la surveillance, le tri et l’application des mises à jour ou modifications de configuration tout au long de la durée de vie de l’application ou du portefeuille.
+## Exemples de scénarios d’attaque
+**Scénario #1 :** Un fournisseur de confiance est compromis par des logiciels malveillants, ce qui entraîne la compromission de vos systèmes informatiques lors de la mise à jour. L’exemple le plus célèbre est probablement : 
+* Le compromis SolarWinds de 2019 qui a conduit à la compromission de ~18 000 organisations. [https://www.npr.org/2021/04/16/985439655/a-worst-nightmare-cyberattack-the-untold-story-of-the-solarwinds-hack] (https://www.npr.org/2021/04/16/985439655/a-worst-nightmare-cyberattack-the-untold-story-of-the-solarwinds-hack)
+**Scénario #2 :** Un fournisseur de confiance est compromis au point de ne se comporter de manière malveillante que dans une condition spécifique. 
+* Le vol de 1,5 milliard de dollars par Bybit en 2025 a été causé par [une attaque de chaîne d’approvisionnement dans un logiciel de portefeuille](https://www.sygnia.co/blog/sygnia-investigation-bybit-hack/) qui ne s’est exécutée que lorsque le portefeuille cible était utilisé. 
+**Scénario #3 :** L’attaque de chaîne d’approvisionnement ['Shai-Hulud'](https://www.cisa.gov/news-events/alerts/2025/09/23/widespread-supply-chain-compromise-impacting-npm-ecosystem) en 2025 a été le premier ver npm auto-propagant réussi. Les attaques ont semé des versions malveillantes de paquets populaires, qui utilisaient un script post-installation pour récolter et exfiltrer des données sensibles vers des dépôts publics GitHub. Le malware détectait également les jetons npm dans l’environnement victime et les utilisait automatiquement pour diffuser des versions malveillantes de tout package accessible. Le ver a atteint plus de 500 versions de paquets avant d’être perturbé par npm. Cette attaque de chaîne d’approvisionnement était avancée, se propageait rapidement et causait des dommages, et en ciblant les machines développeurs, elle a démontré que les développeurs eux-mêmes sont désormais des cibles principales pour les attaques de la chaîne d’approvisionnement. 
+**Scénario #4 :** Les composants fonctionnent généralement avec les mêmes privilèges que l’application elle-même, donc des défauts dans n’importe quel composant peuvent avoir un impact sérieux. Ces défauts peuvent être accidentels (par exemple, une erreur de codage) ou intentionnels (par exemple, une porte dérobée dans un composant). Voici quelques exemples de vulnérabilités exploitables de composants découverts : 
+* CVE-2017-5638, une vulnérabilité d’exécution de code à distance Struts 2 qui permet l’exécution de code arbitraire sur le serveur, a été tenue responsable de violations importantes. 
+* CVE-2021-44228 (« Log4Shell »), une vulnérabilité zero-day d’exécution de code à distance Apache Log4j, a été tenue responsable de campagnes de ransomware, de cryptominage et d’autres attaques. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A03_2025-Software_Supply_Chain_Failures/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;39
+   &lt;/td&gt;
+   &lt;td&gt;22,18 % 
+   &lt;/td&gt;
+   &lt;td&gt;1,86 % 
+   &lt;/td&gt;
+   &lt;td&gt;88,76 % 
+   &lt;/td&gt;
+   &lt;td&gt;35,18 % 
+   &lt;/td&gt;
+   &lt;td&gt;6,96
+   &lt;/td&gt;
+   &lt;td&gt;4,05
+   &lt;/td&gt;
+   &lt;td&gt;729 882
+   &lt;/td&gt;
+   &lt;td&gt;7 647
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+* Établir et utiliser un cycle de développement sécurisé avec des professionnels AppSec pour aider à évaluer et concevoir des contrôles liés à la sécurité et à la confidentialité
+* Établir et utiliser une bibliothèque de modèles de conception sécurisés ou de composants de routes pavées
+* Utiliser la modélisation des menaces pour des parties critiques de l’application telles que l’authentification, le contrôle d’accès, la logique métier et les flux de clés
+* Utiliser la modélisation des menaces comme outil éducatif pour générer un état d’esprit de sécurité
+* Intégrer le langage de sécurité et les contrôles dans les histoires utilisateur
+* Intégrer des vérifications de plausibilité à chaque niveau de votre application (du frontend au backend)
+* Écrire des tests unitaires et d’intégration pour valider que tous les flux critiques sont résistants au modèle de menace. Compiler les cas d’utilisation *et* les cas d’utilisation inappropriés pour chaque niveau de votre application. 
+* Séparer les couches de niveaux sur le système et les couches réseau, en fonction des besoins d’exposition et de protection
+* Séparer les locataires de manière rigoureuse par conception sur tous les niveaux
+## Exemples de scénarios d’attaque
+**Scénario #1 :** Un flux de travail de récupération d’identifiants peut inclure des « questions et réponses », ce qui est interdit par le NIST 800-63b, l’OWASP ASVS et le OWASP Top 10. Les questions et réponses ne peuvent pas être dignes de confiance comme preuve d’identité, car plus d’une personne peut connaître les réponses. De telles fonctionnalités doivent être supprimées et remplacées par une conception plus sécurisée. 
+**Scénario #2 :** Une chaîne de cinémas permet des réductions de réservation de groupe et compte un maximum de quinze participants avant de devoir payer un acompte. Les attaquants pourraient modéliser ce flux de menaces et tester s’ils peuvent trouver un vecteur d’attaque dans la logique métier de l’application, par exemple réserver six cents sièges et tous les cinémas en même temps en quelques requêtes, entraînant une perte massive de revenus. 
+**Scénario #3 :** Le site e-commerce d’une chaîne de distribution ne dispose pas de protection contre les bots gérés par des revendeurs achetant des cartes vidéo haut de gamme pour les revendre sur des sites d’enchères. Cela crée une mauvaise publicité pour les fabricants de cartes vidéo et les propriétaires de chaînes de détail, et endure des tensions avec les passionnés qui ne peuvent obtenir ces cartes à aucun prix. Des règles strictes de conception anti-bots et de logique de domaine, comme les achats effectués dans quelques secondes de disponibilité, peuvent identifier des achats inauthentiques et rejeter ces transactions. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A06_2025-Insecure_Design/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;5
+   &lt;/td&gt;
+   &lt;td&gt;11,33 % 
+   &lt;/td&gt;
+   &lt;td&gt;3,91 % 
+   &lt;/td&gt;
+   &lt;td&gt;85,96 % 
+   &lt;/td&gt;
+   &lt;td&gt;46,48 % 
+   &lt;/td&gt;
+   &lt;td&gt;7.19
+   &lt;/td&gt;
+   &lt;td&gt;2,65
+   &lt;/td&gt;
+   &lt;td&gt;260 288
+   &lt;/td&gt;
+   &lt;td&gt;723
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+Les développeurs doivent implémenter certains ou tous les contrôles suivants, selon le risque de l’application : 
+* S’assurer que toutes les défaillances de connexion, de contrôle d’accès et de validation d’entrée côté serveur peuvent être enregistrées avec suffisamment de contexte utilisateur pour identifier les comptes suspects ou malveillants et conservées suffisamment longtemps pour permettre une analyse médico-légale retardée. 
+* Assurez-vous que chaque partie de votre application contenant un contrôle de sécurité est enregistrée, qu’elle réussisse ou non. 
+* S’assurer que les journaux sont générés dans un format que les solutions de gestion des journaux peuvent facilement consommer. 
+* S’assurer que les données de journal sont correctement encodées pour éviter les injections ou attaques sur les systèmes de journalisation ou de surveillance. 
+* Veiller à ce que toutes les transactions disposent d’une trace d’audit avec des contrôles d’intégrité pour éviter toute altération ou suppression, comme des tables de base de données à ajout uniquement ou autres. 
+* Assurez-vous que toutes les transactions qui génèrent une erreur soient annulées et recommencées. Échouez toujours à la clôture. 
+* Si votre application ou ses utilisateurs se comportent de manière suspecte, lancez une alerte. Créez des conseils pour vos développeurs sur ce sujet afin qu’ils puissent coder contre cela ou acheter un système pour cela. 
+* Les équipes DevSecOps et de sécurité doivent établir des cas d’utilisation efficaces de surveillance et d’alerte, y compris des playbooks afin que les activités suspectes soient détectées et traitées rapidement par l’équipe du Centre des Opérations de Sécurité (SOC). 
+* Ajoutez des « honeytokens » comme pièges pour les attaquants dans votre application, par exemple dans la base de données, les données, comme identité utilisateur réelle et/ou technique. Comme ils ne sont pas utilisés dans les affaires normales, tout accès génère des données de journalisation pouvant être alertées avec presque aucun faux positif. 
+* L’analyse comportementale et le support de l’IA pourraient être optionnellement une technique supplémentaire pour supporter de faibles taux de faux positifs lors des alertes. 
+* Établir ou adopter un plan de réponse et de rétablissement aux incidents, tel que le National Institute of Standards and Technology (NIST) 800-61r2 ou ultérieur. Enseignez à vos développeurs logiciels à quoi ressemblent les attaques et incidents d’applications, afin qu’ils puissent les signaler. 
+Il existe des produits commerciaux et open source de protection d’applications tels que le Mod Security Core Rule Set OWASP, ainsi que des logiciels open source de corrélation de journaux, tels que la pile Elasticsearch, Logstash, Kibana (ELK), qui proposent des tableaux de bord personnalisés et des alertes pouvant vous aider à lutter contre ces problèmes. Il existe également des outils commerciaux d’observabilité qui peuvent vous aider à répondre ou bloquer des attaques en temps quasi réel.
+## Exemples de scénarios d’attaque
+**Scénario #1 :** L’opérateur du site web d’un fournisseur de régime de santé pour enfants n’a pas pu détecter une violation en raison d’un manque de surveillance et de registration. Une partie externe a informé le prestataire du régime de santé qu’un attaquant avait accédé et modifié des milliers de dossiers médicaux sensibles de plus de 3,5 millions d’enfants. Une revue post-incident a révélé que les développeurs du site n’avaient pas corrigé de vulnérabilités significatives. Comme il n’y avait ni journalisation ni surveillance du système, la violation de données pouvait être en cours depuis 2013, soit plus de sept ans. 
+**Scénario #2 :** Une grande compagnie aérienne indienne a subi une violation de données impliquant plus de dix ans de données personnelles de millions de passagers, y compris des données de passeports et de cartes de crédit. La violation de données s’est produite chez un fournisseur tiers d’hébergement cloud, qui a informé la compagnie aérienne après un certain temps. 
+**Scénario #3 :** Une grande compagnie aérienne européenne a subi une violation déclarable selon le RGPD. La violation aurait été causée par des vulnérabilités de sécurité des applications de paiement exploitées par des attaquants, qui ont collecté plus de 400 000 relevés de paiement clients. La compagnie aérienne a été condamnée à une amende de 20 millions de livres sterling par le régulateur de la vie privée. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A09_2025-Security_Logging_and_Alerting_Failures/</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7960,9 +8631,18 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -7979,7 +8659,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -8013,31 +8693,900 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="39">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -8048,6 +9597,49 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F4F4D3D0-A75A-471A-9225-F8FBA886F341}" name="Tableau1" displayName="Tableau1" ref="A1:AH11" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="37" tableBorderDxfId="38" totalsRowBorderDxfId="36">
+  <autoFilter ref="A1:AH11" xr:uid="{F4F4D3D0-A75A-471A-9225-F8FBA886F341}"/>
+  <tableColumns count="34">
+    <tableColumn id="1" xr3:uid="{20C696B3-F3A9-4D52-B31D-9D8663D1DB71}" name="ref_id" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{17243304-7DCB-4BF7-9986-F4AD97FC78CA}" name="name" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{8B25493F-0F71-4BFE-85D4-F5984D21AC75}" name="description" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{F56F0116-19FC-4FCD-A303-1A21A8C96E11}" name="annotation" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{3D791354-91A9-4E1D-BEF6-A9A5A8A22998}" name="name[fr]" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{D8DCB7EE-CBDD-49D5-9BD8-2FDCA39C2393}" name="description[fr]" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{B3212763-7D29-4002-9509-0ADAB8E947E0}" name="annotation[fr]" dataDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{97365EF5-4239-4299-8A88-4B94639A030B}" name="name[cs]" dataDxfId="28"/>
+    <tableColumn id="9" xr3:uid="{9332F77D-1BDC-4F84-9FFD-52FAAB99C0D6}" name="description[cs]" dataDxfId="27"/>
+    <tableColumn id="10" xr3:uid="{259AA177-2D77-4278-8FBC-668F9B2E632E}" name="annotation[cs]" dataDxfId="26"/>
+    <tableColumn id="11" xr3:uid="{56D7B82C-687D-409F-BDAD-82FB932587E2}" name="name[de]" dataDxfId="25"/>
+    <tableColumn id="12" xr3:uid="{923C63BC-ED04-4B8A-A8B2-62773BBB809C}" name="description[de]" dataDxfId="24"/>
+    <tableColumn id="13" xr3:uid="{3AC976CC-F767-49B0-9D10-C0E5E8BE141B}" name="annotation[de]" dataDxfId="23"/>
+    <tableColumn id="14" xr3:uid="{6173A9C3-34B7-428E-B72A-37056E1C1EBD}" name="name[es]" dataDxfId="22"/>
+    <tableColumn id="15" xr3:uid="{8D73EF1A-F638-4F88-B122-97E698A8F65C}" name="description[es]" dataDxfId="21"/>
+    <tableColumn id="16" xr3:uid="{D5227CA4-120B-4DB8-A829-E6A25EA72E35}" name="annotation[es]" dataDxfId="20"/>
+    <tableColumn id="17" xr3:uid="{001384B1-5401-40FC-B7BC-8DAAD7B8ED9C}" name="name[fa]" dataDxfId="19"/>
+    <tableColumn id="18" xr3:uid="{366720CD-3CB7-4463-8EAB-99966D51FFE4}" name="description[fa]" dataDxfId="18"/>
+    <tableColumn id="19" xr3:uid="{120801F2-CF30-48AF-95EB-A5FE039DC1D9}" name="annotation[fa]" dataDxfId="17"/>
+    <tableColumn id="20" xr3:uid="{1B122668-F94F-4389-9D8D-AF7A2AD03138}" name="name[it]" dataDxfId="16"/>
+    <tableColumn id="21" xr3:uid="{591B41BA-0086-434F-9574-480FAD5AB0EE}" name="description[it]" dataDxfId="15"/>
+    <tableColumn id="22" xr3:uid="{DBB49242-33A4-4CE6-8CDC-78B1BD2F8FEB}" name="annotation[it]" dataDxfId="14"/>
+    <tableColumn id="23" xr3:uid="{6BDA09A6-219F-4E16-8511-3587DB546C6D}" name="name[ja]" dataDxfId="13"/>
+    <tableColumn id="24" xr3:uid="{36F23F53-D49E-42CC-8CA2-B27DC821694D}" name="description[ja]" dataDxfId="12"/>
+    <tableColumn id="25" xr3:uid="{3039A195-B467-4670-9FA1-5C386D80016E}" name="annotation[ja]" dataDxfId="11"/>
+    <tableColumn id="26" xr3:uid="{E0AC4B3E-211E-472C-9504-4AEDFF7647EC}" name="name[ko]" dataDxfId="10"/>
+    <tableColumn id="27" xr3:uid="{A7ED36D1-478D-434A-BEE9-093D928BC94F}" name="description[ko]" dataDxfId="9"/>
+    <tableColumn id="28" xr3:uid="{AC28BFD9-D5BE-40D9-81E4-E43731706E28}" name="annotation[ko]" dataDxfId="8"/>
+    <tableColumn id="29" xr3:uid="{0C382B30-4F63-4555-994F-52EA358D7FCE}" name="name[pt]" dataDxfId="7"/>
+    <tableColumn id="30" xr3:uid="{750FC0D5-9907-4470-8CFC-AC612C3999FE}" name="description[pt]" dataDxfId="6"/>
+    <tableColumn id="31" xr3:uid="{E340CC54-AE05-44BA-88C2-7E381DA7CAA2}" name="annotation[pt]" dataDxfId="5"/>
+    <tableColumn id="32" xr3:uid="{8EDE774A-6638-496F-9CE5-7270A55EFEC3}" name="name[zh]" dataDxfId="4"/>
+    <tableColumn id="33" xr3:uid="{13B7C29B-1ADE-4CA4-9203-3612E8567D23}" name="description[zh]" dataDxfId="3"/>
+    <tableColumn id="34" xr3:uid="{6B4F0FB1-ECB4-4D63-B0EE-75B41FA57863}" name="annotation[zh]" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8350,8 +9942,8 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4"/>
-      <c r="E1" s="5" t="s">
+      <c r="D1" s="2"/>
+      <c r="E1" s="3" t="s">
         <v>366</v>
       </c>
     </row>
@@ -8663,1131 +10255,1154 @@
     <col min="34" max="34" width="120" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:34" s="18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="Z1" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AA1" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AB1" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AC1" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AD1" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AE1" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AF1" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AG1" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AH1" s="17" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>367</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1" t="s">
+      <c r="G2" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="M2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="N2" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="O2" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="P2" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="Q2" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="R2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="S2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="T2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="U2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="V2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="W2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="X2" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="Y2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="Z2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AA2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="AB2" s="1" t="s">
+      <c r="AB2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="AC2" s="1" t="s">
+      <c r="AC2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="AD2" s="1" t="s">
+      <c r="AD2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="AE2" s="1" t="s">
+      <c r="AE2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="AF2" s="1" t="s">
+      <c r="AF2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="AG2" s="1" t="s">
+      <c r="AG2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="AH2" s="1" t="s">
+      <c r="AH2" s="8" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1" t="s">
+      <c r="G3" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="M3" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="N3" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="O3" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="P3" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="Q3" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="R3" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="S3" s="1" t="s">
+      <c r="S3" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="T3" s="1" t="s">
+      <c r="T3" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="U3" s="1" t="s">
+      <c r="U3" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="V3" s="1" t="s">
+      <c r="V3" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="W3" s="1" t="s">
+      <c r="W3" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="X3" s="1" t="s">
+      <c r="X3" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="Y3" s="1" t="s">
+      <c r="Y3" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="Z3" s="1" t="s">
+      <c r="Z3" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="AA3" s="1" t="s">
+      <c r="AA3" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="AB3" s="1" t="s">
+      <c r="AB3" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="AC3" s="1" t="s">
+      <c r="AC3" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="AD3" s="1" t="s">
+      <c r="AD3" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="AE3" s="1" t="s">
+      <c r="AE3" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="AF3" s="1" t="s">
+      <c r="AF3" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="AG3" s="1" t="s">
+      <c r="AG3" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="AH3" s="1" t="s">
+      <c r="AH3" s="8" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1" t="s">
+      <c r="G4" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="L4" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="M4" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="N4" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="O4" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="P4" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="Q4" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="R4" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="S4" s="1" t="s">
+      <c r="S4" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="T4" s="1" t="s">
+      <c r="T4" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="U4" s="1" t="s">
+      <c r="U4" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="V4" s="1" t="s">
+      <c r="V4" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="W4" s="1" t="s">
+      <c r="W4" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="X4" s="1" t="s">
+      <c r="X4" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="Y4" s="1" t="s">
+      <c r="Y4" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="Z4" s="1" t="s">
+      <c r="Z4" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="AA4" s="1" t="s">
+      <c r="AA4" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="AB4" s="1" t="s">
+      <c r="AB4" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="AC4" s="1" t="s">
+      <c r="AC4" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="AD4" s="1" t="s">
+      <c r="AD4" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="AE4" s="1" t="s">
+      <c r="AE4" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="AF4" s="1" t="s">
+      <c r="AF4" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="AG4" s="1" t="s">
+      <c r="AG4" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="AH4" s="1" t="s">
+      <c r="AH4" s="8" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1" t="s">
+      <c r="G5" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="L5" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="M5" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="N5" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="O5" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="P5" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="Q5" s="1" t="s">
+      <c r="Q5" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="R5" s="1" t="s">
+      <c r="R5" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="S5" s="1" t="s">
+      <c r="S5" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="T5" s="1" t="s">
+      <c r="T5" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="U5" s="1" t="s">
+      <c r="U5" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="V5" s="1" t="s">
+      <c r="V5" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="W5" s="1" t="s">
+      <c r="W5" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="X5" s="1" t="s">
+      <c r="X5" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="Y5" s="1" t="s">
+      <c r="Y5" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="Z5" s="1" t="s">
+      <c r="Z5" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="AA5" s="1" t="s">
+      <c r="AA5" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="AB5" s="1" t="s">
+      <c r="AB5" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="AC5" s="1" t="s">
+      <c r="AC5" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="AD5" s="1" t="s">
+      <c r="AD5" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="AE5" s="1" t="s">
+      <c r="AE5" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="AF5" s="1" t="s">
+      <c r="AF5" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="AG5" s="1" t="s">
+      <c r="AG5" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="AH5" s="1" t="s">
+      <c r="AH5" s="8" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1" t="s">
+      <c r="G6" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="M6" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="N6" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="O6" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="P6" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="Q6" s="1" t="s">
+      <c r="Q6" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="R6" s="1" t="s">
+      <c r="R6" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="S6" s="1" t="s">
+      <c r="S6" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="T6" s="1" t="s">
+      <c r="T6" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="U6" s="1" t="s">
+      <c r="U6" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="V6" s="1" t="s">
+      <c r="V6" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="W6" s="1" t="s">
+      <c r="W6" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="X6" s="1" t="s">
+      <c r="X6" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="Y6" s="1" t="s">
+      <c r="Y6" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="Z6" s="1" t="s">
+      <c r="Z6" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="AA6" s="1" t="s">
+      <c r="AA6" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="AB6" s="1" t="s">
+      <c r="AB6" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="AC6" s="1" t="s">
+      <c r="AC6" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="AD6" s="1" t="s">
+      <c r="AD6" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="AE6" s="1" t="s">
+      <c r="AE6" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="AF6" s="1" t="s">
+      <c r="AF6" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="AG6" s="1" t="s">
+      <c r="AG6" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="AH6" s="1" t="s">
+      <c r="AH6" s="8" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1" t="s">
+      <c r="G7" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L7" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="M7" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="N7" s="1" t="s">
+      <c r="N7" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="O7" s="1" t="s">
+      <c r="O7" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="P7" s="1" t="s">
+      <c r="P7" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="Q7" s="1" t="s">
+      <c r="Q7" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="R7" s="1" t="s">
+      <c r="R7" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="S7" s="1" t="s">
+      <c r="S7" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="T7" s="1" t="s">
+      <c r="T7" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="U7" s="1" t="s">
+      <c r="U7" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="V7" s="1" t="s">
+      <c r="V7" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="W7" s="1" t="s">
+      <c r="W7" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="X7" s="1" t="s">
+      <c r="X7" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="Y7" s="1" t="s">
+      <c r="Y7" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="Z7" s="1" t="s">
+      <c r="Z7" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="AA7" s="1" t="s">
+      <c r="AA7" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="AB7" s="1" t="s">
+      <c r="AB7" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="AC7" s="1" t="s">
+      <c r="AC7" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="AD7" s="1" t="s">
+      <c r="AD7" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="AE7" s="1" t="s">
+      <c r="AE7" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="AF7" s="1" t="s">
+      <c r="AF7" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="AG7" s="1" t="s">
+      <c r="AG7" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="AH7" s="1" t="s">
+      <c r="AH7" s="8" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="8" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1" t="s">
+      <c r="G8" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="L8" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="M8" s="1" t="s">
+      <c r="M8" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="N8" s="1" t="s">
+      <c r="N8" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="O8" s="1" t="s">
+      <c r="O8" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="P8" s="1" t="s">
+      <c r="P8" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="Q8" s="1" t="s">
+      <c r="Q8" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="R8" s="1" t="s">
+      <c r="R8" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="S8" s="1" t="s">
+      <c r="S8" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="T8" s="1" t="s">
+      <c r="T8" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="U8" s="1" t="s">
+      <c r="U8" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="V8" s="1" t="s">
+      <c r="V8" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="W8" s="1" t="s">
+      <c r="W8" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="X8" s="1" t="s">
+      <c r="X8" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="Y8" s="1" t="s">
+      <c r="Y8" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="Z8" s="1" t="s">
+      <c r="Z8" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="AA8" s="1" t="s">
+      <c r="AA8" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="AB8" s="1" t="s">
+      <c r="AB8" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="AC8" s="1" t="s">
+      <c r="AC8" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="AD8" s="1" t="s">
+      <c r="AD8" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="AE8" s="1" t="s">
+      <c r="AE8" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="AF8" s="1" t="s">
+      <c r="AF8" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="AG8" s="1" t="s">
+      <c r="AG8" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="AH8" s="1" t="s">
+      <c r="AH8" s="8" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="7" t="s">
         <v>275</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="5" t="s">
         <v>373</v>
       </c>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1" t="s">
+      <c r="G9" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="K9" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="L9" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="M9" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="N9" s="1" t="s">
+      <c r="N9" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="O9" s="1" t="s">
+      <c r="O9" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="P9" s="1" t="s">
+      <c r="P9" s="4" t="s">
         <v>288</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="Q9" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="R9" s="1" t="s">
+      <c r="R9" s="4" t="s">
         <v>289</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="S9" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="T9" s="1" t="s">
+      <c r="T9" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="U9" s="1" t="s">
+      <c r="U9" s="4" t="s">
         <v>291</v>
       </c>
-      <c r="V9" s="1" t="s">
+      <c r="V9" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="W9" s="1" t="s">
+      <c r="W9" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="X9" s="1" t="s">
+      <c r="X9" s="4" t="s">
         <v>294</v>
       </c>
-      <c r="Y9" s="1" t="s">
+      <c r="Y9" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="Z9" s="1" t="s">
+      <c r="Z9" s="4" t="s">
         <v>296</v>
       </c>
-      <c r="AA9" s="1" t="s">
+      <c r="AA9" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="AB9" s="1" t="s">
+      <c r="AB9" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="AC9" s="1" t="s">
+      <c r="AC9" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="AD9" s="1" t="s">
+      <c r="AD9" s="4" t="s">
         <v>300</v>
       </c>
-      <c r="AE9" s="1" t="s">
+      <c r="AE9" s="4" t="s">
         <v>301</v>
       </c>
-      <c r="AF9" s="1" t="s">
+      <c r="AF9" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="AG9" s="1" t="s">
+      <c r="AG9" s="4" t="s">
         <v>303</v>
       </c>
-      <c r="AH9" s="1" t="s">
+      <c r="AH9" s="8" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="10" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="7" t="s">
         <v>305</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="4" t="s">
         <v>306</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="4" t="s">
         <v>309</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1" t="s">
+      <c r="G10" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>310</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" s="4" t="s">
         <v>311</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="4" t="s">
         <v>312</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="K10" s="4" t="s">
         <v>313</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="L10" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="M10" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="N10" s="1" t="s">
+      <c r="N10" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="O10" s="1" t="s">
+      <c r="O10" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="P10" s="1" t="s">
+      <c r="P10" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="Q10" s="1" t="s">
+      <c r="Q10" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="R10" s="1" t="s">
+      <c r="R10" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="S10" s="1" t="s">
+      <c r="S10" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="T10" s="1" t="s">
+      <c r="T10" s="4" t="s">
         <v>306</v>
       </c>
-      <c r="U10" s="1" t="s">
+      <c r="U10" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="V10" s="1" t="s">
+      <c r="V10" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="W10" s="1" t="s">
+      <c r="W10" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="X10" s="1" t="s">
+      <c r="X10" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="Y10" s="1" t="s">
+      <c r="Y10" s="4" t="s">
         <v>326</v>
       </c>
-      <c r="Z10" s="1" t="s">
+      <c r="Z10" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="AA10" s="1" t="s">
+      <c r="AA10" s="4" t="s">
         <v>328</v>
       </c>
-      <c r="AB10" s="1" t="s">
+      <c r="AB10" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="AC10" s="1" t="s">
+      <c r="AC10" s="4" t="s">
         <v>330</v>
       </c>
-      <c r="AD10" s="1" t="s">
+      <c r="AD10" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="AE10" s="1" t="s">
+      <c r="AE10" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="AF10" s="1" t="s">
+      <c r="AF10" s="4" t="s">
         <v>333</v>
       </c>
-      <c r="AG10" s="1" t="s">
+      <c r="AG10" s="4" t="s">
         <v>334</v>
       </c>
-      <c r="AH10" s="1" t="s">
+      <c r="AH10" s="8" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="11" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="9" t="s">
         <v>336</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="10" t="s">
         <v>338</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="10" t="s">
         <v>339</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="10" t="s">
         <v>340</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="11" t="s">
         <v>375</v>
       </c>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1" t="s">
+      <c r="G11" s="12" t="s">
+        <v>383</v>
+      </c>
+      <c r="H11" s="10" t="s">
         <v>341</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="10" t="s">
         <v>342</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="10" t="s">
         <v>343</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="K11" s="10" t="s">
         <v>344</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="L11" s="10" t="s">
         <v>345</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="M11" s="10" t="s">
         <v>346</v>
       </c>
-      <c r="N11" s="1" t="s">
+      <c r="N11" s="10" t="s">
         <v>347</v>
       </c>
-      <c r="O11" s="1" t="s">
+      <c r="O11" s="10" t="s">
         <v>348</v>
       </c>
-      <c r="P11" s="1" t="s">
+      <c r="P11" s="10" t="s">
         <v>349</v>
       </c>
-      <c r="Q11" s="1" t="s">
+      <c r="Q11" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="R11" s="1" t="s">
+      <c r="R11" s="10" t="s">
         <v>350</v>
       </c>
-      <c r="S11" s="1" t="s">
+      <c r="S11" s="10" t="s">
         <v>351</v>
       </c>
-      <c r="T11" s="1" t="s">
+      <c r="T11" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="U11" s="1" t="s">
+      <c r="U11" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="V11" s="1" t="s">
+      <c r="V11" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="W11" s="1" t="s">
+      <c r="W11" s="10" t="s">
         <v>354</v>
       </c>
-      <c r="X11" s="1" t="s">
+      <c r="X11" s="10" t="s">
         <v>355</v>
       </c>
-      <c r="Y11" s="1" t="s">
+      <c r="Y11" s="10" t="s">
         <v>356</v>
       </c>
-      <c r="Z11" s="1" t="s">
+      <c r="Z11" s="10" t="s">
         <v>357</v>
       </c>
-      <c r="AA11" s="1" t="s">
+      <c r="AA11" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="AB11" s="1" t="s">
+      <c r="AB11" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="AC11" s="1" t="s">
+      <c r="AC11" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="AD11" s="1" t="s">
+      <c r="AD11" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="AE11" s="1" t="s">
+      <c r="AE11" s="10" t="s">
         <v>362</v>
       </c>
-      <c r="AF11" s="1" t="s">
+      <c r="AF11" s="10" t="s">
         <v>363</v>
       </c>
-      <c r="AG11" s="1" t="s">
+      <c r="AG11" s="10" t="s">
         <v>364</v>
       </c>
-      <c r="AH11" s="1" t="s">
+      <c r="AH11" s="13" t="s">
         <v>365</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[Excel+YAML] Update Excel version of OWASP Top 10 Web 2025 + Update YAML
Fix & Simplify URNs
</commit_message>
<xml_diff>
--- a/tools/excel/owasp/owasp-top-10-web_2025.xlsx
+++ b/tools/excel/owasp/owasp-top-10-web_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\owasp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F5AF1F-7CFE-4CA5-8CC4-7BED21A95881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FFADF6E-28B9-4AB5-BBFD-DF0876D2B2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30696" yWindow="-9720" windowWidth="22824" windowHeight="16344" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="398">
   <si>
     <t>type</t>
   </si>
@@ -202,9 +202,6 @@
   </si>
   <si>
     <t>base_urn</t>
-  </si>
-  <si>
-    <t>urn:intuitem:risk:owasp-top-10-web_2025</t>
   </si>
   <si>
     <t>annotation</t>
@@ -8617,6 +8614,42 @@
 **Scénario #3 :** Une grande compagnie aérienne européenne a subi une violation déclarable selon le RGPD. La violation aurait été causée par des vulnérabilités de sécurité des applications de paiement exploitées par des attaquants, qui ont collecté plus de 400 000 relevés de paiement clients. La compagnie aérienne a été condamnée à une amende de 20 millions de livres sterling par le régulateur de la vie privée. 
 Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A09_2025-Security_Logging_and_Alerting_Failures/</t>
   </si>
+  <si>
+    <t>urn:intuitem:risk:threat:owasp-top-10-web_2025</t>
+  </si>
+  <si>
+    <t>node_id</t>
+  </si>
+  <si>
+    <t>A01</t>
+  </si>
+  <si>
+    <t>A02</t>
+  </si>
+  <si>
+    <t>A03</t>
+  </si>
+  <si>
+    <t>A04</t>
+  </si>
+  <si>
+    <t>A05</t>
+  </si>
+  <si>
+    <t>A06</t>
+  </si>
+  <si>
+    <t>A07</t>
+  </si>
+  <si>
+    <t>A08</t>
+  </si>
+  <si>
+    <t>A09</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
 </sst>
 </file>
 
@@ -8645,7 +8678,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -8658,8 +8691,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor theme="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor theme="0" tint="-0.14999847407452621"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -8697,57 +8742,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -8755,12 +8750,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <left/>
+      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -8772,9 +8763,7 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -8782,14 +8771,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8798,48 +8788,29 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="39">
+  <dxfs count="38">
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -8849,27 +8820,11 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <scheme val="none"/>
+        <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -8880,534 +8835,860 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <fill>
         <patternFill patternType="solid">
@@ -9420,20 +9701,32 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -9445,129 +9738,203 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
+        <left style="thin">
           <color indexed="64"/>
-        </right>
+        </left>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border outline="0">
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -9586,6 +9953,60 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="1"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -9600,43 +10021,44 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F4F4D3D0-A75A-471A-9225-F8FBA886F341}" name="Tableau1" displayName="Tableau1" ref="A1:AH11" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="37" tableBorderDxfId="38" totalsRowBorderDxfId="36">
-  <autoFilter ref="A1:AH11" xr:uid="{F4F4D3D0-A75A-471A-9225-F8FBA886F341}"/>
-  <tableColumns count="34">
-    <tableColumn id="1" xr3:uid="{20C696B3-F3A9-4D52-B31D-9D8663D1DB71}" name="ref_id" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{17243304-7DCB-4BF7-9986-F4AD97FC78CA}" name="name" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{8B25493F-0F71-4BFE-85D4-F5984D21AC75}" name="description" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{F56F0116-19FC-4FCD-A303-1A21A8C96E11}" name="annotation" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{3D791354-91A9-4E1D-BEF6-A9A5A8A22998}" name="name[fr]" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{D8DCB7EE-CBDD-49D5-9BD8-2FDCA39C2393}" name="description[fr]" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{B3212763-7D29-4002-9509-0ADAB8E947E0}" name="annotation[fr]" dataDxfId="29"/>
-    <tableColumn id="8" xr3:uid="{97365EF5-4239-4299-8A88-4B94639A030B}" name="name[cs]" dataDxfId="28"/>
-    <tableColumn id="9" xr3:uid="{9332F77D-1BDC-4F84-9FFD-52FAAB99C0D6}" name="description[cs]" dataDxfId="27"/>
-    <tableColumn id="10" xr3:uid="{259AA177-2D77-4278-8FBC-668F9B2E632E}" name="annotation[cs]" dataDxfId="26"/>
-    <tableColumn id="11" xr3:uid="{56D7B82C-687D-409F-BDAD-82FB932587E2}" name="name[de]" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{923C63BC-ED04-4B8A-A8B2-62773BBB809C}" name="description[de]" dataDxfId="24"/>
-    <tableColumn id="13" xr3:uid="{3AC976CC-F767-49B0-9D10-C0E5E8BE141B}" name="annotation[de]" dataDxfId="23"/>
-    <tableColumn id="14" xr3:uid="{6173A9C3-34B7-428E-B72A-37056E1C1EBD}" name="name[es]" dataDxfId="22"/>
-    <tableColumn id="15" xr3:uid="{8D73EF1A-F638-4F88-B122-97E698A8F65C}" name="description[es]" dataDxfId="21"/>
-    <tableColumn id="16" xr3:uid="{D5227CA4-120B-4DB8-A829-E6A25EA72E35}" name="annotation[es]" dataDxfId="20"/>
-    <tableColumn id="17" xr3:uid="{001384B1-5401-40FC-B7BC-8DAAD7B8ED9C}" name="name[fa]" dataDxfId="19"/>
-    <tableColumn id="18" xr3:uid="{366720CD-3CB7-4463-8EAB-99966D51FFE4}" name="description[fa]" dataDxfId="18"/>
-    <tableColumn id="19" xr3:uid="{120801F2-CF30-48AF-95EB-A5FE039DC1D9}" name="annotation[fa]" dataDxfId="17"/>
-    <tableColumn id="20" xr3:uid="{1B122668-F94F-4389-9D8D-AF7A2AD03138}" name="name[it]" dataDxfId="16"/>
-    <tableColumn id="21" xr3:uid="{591B41BA-0086-434F-9574-480FAD5AB0EE}" name="description[it]" dataDxfId="15"/>
-    <tableColumn id="22" xr3:uid="{DBB49242-33A4-4CE6-8CDC-78B1BD2F8FEB}" name="annotation[it]" dataDxfId="14"/>
-    <tableColumn id="23" xr3:uid="{6BDA09A6-219F-4E16-8511-3587DB546C6D}" name="name[ja]" dataDxfId="13"/>
-    <tableColumn id="24" xr3:uid="{36F23F53-D49E-42CC-8CA2-B27DC821694D}" name="description[ja]" dataDxfId="12"/>
-    <tableColumn id="25" xr3:uid="{3039A195-B467-4670-9FA1-5C386D80016E}" name="annotation[ja]" dataDxfId="11"/>
-    <tableColumn id="26" xr3:uid="{E0AC4B3E-211E-472C-9504-4AEDFF7647EC}" name="name[ko]" dataDxfId="10"/>
-    <tableColumn id="27" xr3:uid="{A7ED36D1-478D-434A-BEE9-093D928BC94F}" name="description[ko]" dataDxfId="9"/>
-    <tableColumn id="28" xr3:uid="{AC28BFD9-D5BE-40D9-81E4-E43731706E28}" name="annotation[ko]" dataDxfId="8"/>
-    <tableColumn id="29" xr3:uid="{0C382B30-4F63-4555-994F-52EA358D7FCE}" name="name[pt]" dataDxfId="7"/>
-    <tableColumn id="30" xr3:uid="{750FC0D5-9907-4470-8CFC-AC612C3999FE}" name="description[pt]" dataDxfId="6"/>
-    <tableColumn id="31" xr3:uid="{E340CC54-AE05-44BA-88C2-7E381DA7CAA2}" name="annotation[pt]" dataDxfId="5"/>
-    <tableColumn id="32" xr3:uid="{8EDE774A-6638-496F-9CE5-7270A55EFEC3}" name="name[zh]" dataDxfId="4"/>
-    <tableColumn id="33" xr3:uid="{13B7C29B-1ADE-4CA4-9203-3612E8567D23}" name="description[zh]" dataDxfId="3"/>
-    <tableColumn id="34" xr3:uid="{6B4F0FB1-ECB4-4D63-B0EE-75B41FA57863}" name="annotation[zh]" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A014C139-48ED-459E-8EFE-0F48BB944E29}" name="Tableau1" displayName="Tableau1" ref="A1:AI11" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36" tableBorderDxfId="35">
+  <autoFilter ref="A1:AI11" xr:uid="{A014C139-48ED-459E-8EFE-0F48BB944E29}"/>
+  <tableColumns count="35">
+    <tableColumn id="1" xr3:uid="{25AE8D30-3860-4111-8EA6-C4C7AEECC6EB}" name="ref_id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{92E23933-32F2-41EA-BF91-455565D13AFD}" name="node_id" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{CD524151-5700-4186-A8E3-1B3BECA35D31}" name="name" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{0BFFD00C-098B-4E57-A16B-3C376911F0A6}" name="description" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{1031B7B0-FAC6-47EA-BF11-B9A35519FBFD}" name="annotation" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{FB68E663-983D-432F-8C12-C673829B1EE9}" name="name[fr]" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{E7898F1E-1574-4B4E-A4FD-758820DEADE4}" name="description[fr]" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{3CA9968D-8F68-4C21-95A2-FFD6FC8B7493}" name="annotation[fr]" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{93E9EC66-775C-4641-BD7A-A06C2F9D56B2}" name="name[cs]" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{51366F19-9468-42E8-90A9-B9C23225D7DD}" name="description[cs]" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{8C2133FF-64CE-4C7C-AEC1-7AFB9456E6CF}" name="annotation[cs]" dataDxfId="24"/>
+    <tableColumn id="12" xr3:uid="{DEA91A07-6088-4648-BC99-DBBE4BB97527}" name="name[de]" dataDxfId="23"/>
+    <tableColumn id="13" xr3:uid="{AB6F2498-4869-43FA-92E5-0EDAFE791BAD}" name="description[de]" dataDxfId="22"/>
+    <tableColumn id="14" xr3:uid="{39519832-5547-4B8D-8CE3-A5F59F22EBAC}" name="annotation[de]" dataDxfId="21"/>
+    <tableColumn id="15" xr3:uid="{8460DD8D-47C6-4E87-AD01-F3AD20769748}" name="name[es]" dataDxfId="20"/>
+    <tableColumn id="16" xr3:uid="{5EAA485E-15DE-46C4-A9D2-97C138336F35}" name="description[es]" dataDxfId="19"/>
+    <tableColumn id="17" xr3:uid="{B3866A17-8967-4C4E-A5EE-56274B48C1F1}" name="annotation[es]" dataDxfId="18"/>
+    <tableColumn id="18" xr3:uid="{CC115383-C845-4A5F-BAF5-C6ABAC7C4E12}" name="name[fa]" dataDxfId="17"/>
+    <tableColumn id="19" xr3:uid="{552DBEA8-469F-4D67-9E2E-98218233E662}" name="description[fa]" dataDxfId="16"/>
+    <tableColumn id="20" xr3:uid="{31BF1538-369A-4B29-B01B-CB8C16854DB5}" name="annotation[fa]" dataDxfId="15"/>
+    <tableColumn id="21" xr3:uid="{5D79E7BE-5B52-46D7-B7A5-6104BC1A1D44}" name="name[it]" dataDxfId="14"/>
+    <tableColumn id="22" xr3:uid="{C8923F58-6252-4E60-AC02-E32CBC8BC741}" name="description[it]" dataDxfId="13"/>
+    <tableColumn id="23" xr3:uid="{F48E3656-A969-4E25-A065-330F8D08E7D2}" name="annotation[it]" dataDxfId="12"/>
+    <tableColumn id="24" xr3:uid="{32FDE793-892B-41C0-87A4-EE72BF642E10}" name="name[ja]" dataDxfId="11"/>
+    <tableColumn id="25" xr3:uid="{499C9F0B-0066-4FFD-B117-F2A167ABAA64}" name="description[ja]" dataDxfId="10"/>
+    <tableColumn id="26" xr3:uid="{F30E2A0D-2E40-4166-858A-B03C02C9B7E6}" name="annotation[ja]" dataDxfId="9"/>
+    <tableColumn id="27" xr3:uid="{9DFEFF6B-B495-4084-AF12-32844FFE1E6D}" name="name[ko]" dataDxfId="8"/>
+    <tableColumn id="28" xr3:uid="{89D67697-85DF-43A7-8ADC-439089931056}" name="description[ko]" dataDxfId="7"/>
+    <tableColumn id="29" xr3:uid="{1FA2710F-4C36-4270-94CF-7E241AC56D9D}" name="annotation[ko]" dataDxfId="6"/>
+    <tableColumn id="30" xr3:uid="{DB1A945B-B6AA-45F9-99F6-19E338C66ABE}" name="name[pt]" dataDxfId="5"/>
+    <tableColumn id="31" xr3:uid="{4044319C-6166-474F-A4F5-EB6FE072A4DA}" name="description[pt]" dataDxfId="4"/>
+    <tableColumn id="32" xr3:uid="{3D009E4C-699E-4946-A3CF-B80EEE277683}" name="annotation[pt]" dataDxfId="3"/>
+    <tableColumn id="33" xr3:uid="{84E7C3A7-8E19-474F-810B-09585BAC9C18}" name="name[zh]" dataDxfId="2"/>
+    <tableColumn id="34" xr3:uid="{891B07E7-E061-4AD2-B36B-74CA005DED85}" name="description[zh]" dataDxfId="1"/>
+    <tableColumn id="35" xr3:uid="{AF75C4F6-F5AB-45F4-A48B-8353C10BDD88}" name="annotation[zh]" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -9944,7 +10366,7 @@
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -10206,7 +10628,7 @@
         <v>51</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>52</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>
@@ -10216,1187 +10638,1221 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AH11"/>
+  <dimension ref="A1:AI11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="3" width="100" customWidth="1"/>
-    <col min="4" max="4" width="120" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="100" customWidth="1"/>
-    <col min="7" max="7" width="120" customWidth="1"/>
-    <col min="8" max="8" width="42" customWidth="1"/>
-    <col min="9" max="9" width="100" customWidth="1"/>
-    <col min="10" max="10" width="120" customWidth="1"/>
-    <col min="11" max="11" width="42" customWidth="1"/>
-    <col min="12" max="12" width="100" customWidth="1"/>
-    <col min="13" max="13" width="120" customWidth="1"/>
-    <col min="14" max="14" width="42" customWidth="1"/>
-    <col min="15" max="15" width="100" customWidth="1"/>
-    <col min="16" max="16" width="120" customWidth="1"/>
-    <col min="17" max="17" width="42" customWidth="1"/>
-    <col min="18" max="18" width="100" customWidth="1"/>
-    <col min="19" max="19" width="120" customWidth="1"/>
-    <col min="20" max="20" width="42" customWidth="1"/>
-    <col min="21" max="21" width="100" customWidth="1"/>
-    <col min="22" max="22" width="120" customWidth="1"/>
-    <col min="23" max="23" width="42" customWidth="1"/>
-    <col min="24" max="24" width="100" customWidth="1"/>
-    <col min="25" max="25" width="120" customWidth="1"/>
-    <col min="26" max="26" width="42" customWidth="1"/>
-    <col min="27" max="27" width="100" customWidth="1"/>
-    <col min="28" max="28" width="120" customWidth="1"/>
-    <col min="29" max="29" width="42" customWidth="1"/>
-    <col min="30" max="30" width="100" customWidth="1"/>
-    <col min="31" max="31" width="120" customWidth="1"/>
-    <col min="32" max="32" width="42" customWidth="1"/>
-    <col min="33" max="33" width="100" customWidth="1"/>
-    <col min="34" max="34" width="120" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="4" max="4" width="100" customWidth="1"/>
+    <col min="5" max="5" width="120" customWidth="1"/>
+    <col min="6" max="6" width="42" customWidth="1"/>
+    <col min="7" max="7" width="100" customWidth="1"/>
+    <col min="8" max="8" width="120" customWidth="1"/>
+    <col min="9" max="9" width="42" customWidth="1"/>
+    <col min="10" max="10" width="100" customWidth="1"/>
+    <col min="11" max="11" width="120" customWidth="1"/>
+    <col min="12" max="12" width="42" customWidth="1"/>
+    <col min="13" max="13" width="100" customWidth="1"/>
+    <col min="14" max="14" width="120" customWidth="1"/>
+    <col min="15" max="15" width="42" customWidth="1"/>
+    <col min="16" max="16" width="100" customWidth="1"/>
+    <col min="17" max="17" width="120" customWidth="1"/>
+    <col min="18" max="18" width="42" customWidth="1"/>
+    <col min="19" max="19" width="100" customWidth="1"/>
+    <col min="20" max="20" width="120" customWidth="1"/>
+    <col min="21" max="21" width="42" customWidth="1"/>
+    <col min="22" max="22" width="100" customWidth="1"/>
+    <col min="23" max="23" width="120" customWidth="1"/>
+    <col min="24" max="24" width="42" customWidth="1"/>
+    <col min="25" max="25" width="100" customWidth="1"/>
+    <col min="26" max="26" width="120" customWidth="1"/>
+    <col min="27" max="27" width="42" customWidth="1"/>
+    <col min="28" max="28" width="100" customWidth="1"/>
+    <col min="29" max="29" width="120" customWidth="1"/>
+    <col min="30" max="30" width="42" customWidth="1"/>
+    <col min="31" max="31" width="100" customWidth="1"/>
+    <col min="32" max="32" width="120" customWidth="1"/>
+    <col min="33" max="33" width="42" customWidth="1"/>
+    <col min="34" max="34" width="100" customWidth="1"/>
+    <col min="35" max="35" width="120" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="18" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:35" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="D1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="E1" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="16" t="s">
+      <c r="I1" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="I1" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="J1" s="15" t="s">
+      <c r="L1" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="K1" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="L1" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="15" t="s">
+      <c r="O1" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="P1" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="N1" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="O1" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="P1" s="15" t="s">
+      <c r="R1" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="S1" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="T1" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="Q1" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="R1" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="S1" s="15" t="s">
+      <c r="U1" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="V1" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="W1" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="T1" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="U1" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="V1" s="15" t="s">
+      <c r="X1" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y1" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z1" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="W1" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="X1" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y1" s="15" t="s">
+      <c r="AA1" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB1" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC1" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="Z1" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA1" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="AB1" s="15" t="s">
+      <c r="AD1" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AE1" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="AF1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="AC1" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="AD1" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="AE1" s="15" t="s">
+      <c r="AG1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="AH1" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="AF1" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="AG1" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="AH1" s="17" t="s">
+    </row>
+    <row r="2" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
         <v>63</v>
       </c>
+      <c r="B2" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y2" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="Z2" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA2" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="AC2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD2" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE2" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="AF2" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="AG2" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="AH2" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="AI2" s="5" t="s">
+        <v>93</v>
+      </c>
     </row>
-    <row r="2" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F2" s="5" t="s">
+    <row r="3" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="H3" s="7" t="s">
         <v>377</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="T2" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="U2" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="V2" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="W2" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="X2" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="Y2" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="Z2" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="AA2" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AB2" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="AC2" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD2" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="AE2" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="AF2" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="AG2" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="AH2" s="8" t="s">
-        <v>94</v>
+      <c r="I3" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="P3" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q3" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="R3" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="S3" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="T3" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="U3" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V3" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="W3" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="X3" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="Y3" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z3" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="AA3" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="AB3" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="AC3" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="AD3" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="AE3" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF3" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="AG3" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="AH3" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="AI3" s="8" t="s">
+        <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="F3" s="5" t="s">
+    <row r="4" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H4" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="AC4" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="AD4" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="AE4" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="AF4" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="AG4" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="AH4" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="AI4" s="5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>378</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="R3" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="U3" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="Y3" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="AA3" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="AB3" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="AC3" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="AD3" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="AE3" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="AF3" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="AG3" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="AH3" s="8" t="s">
-        <v>125</v>
+      <c r="I5" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="R5" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="S5" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="T5" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="U5" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="V5" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="W5" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="X5" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="Y5" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="Z5" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="AA5" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="AB5" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC5" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="AD5" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="AE5" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="AF5" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG5" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="AH5" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="AI5" s="8" t="s">
+        <v>184</v>
       </c>
     </row>
-    <row r="4" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="G4" s="6" t="s">
+    <row r="6" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="U6" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="AB6" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="AC6" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="AD6" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="AE6" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="AF6" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="AG6" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="AH6" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="AI6" s="5" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="H7" s="7" t="s">
         <v>384</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="N4" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="O4" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q4" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="R4" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="S4" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="T4" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="U4" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="V4" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="W4" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="X4" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="Y4" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="Z4" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA4" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="AB4" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="AC4" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="AD4" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="AE4" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="AF4" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="AG4" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="AH4" s="8" t="s">
-        <v>154</v>
+      <c r="I7" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="N7" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="P7" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q7" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="R7" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="S7" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="T7" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="U7" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="V7" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="W7" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="X7" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="Y7" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="Z7" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="AA7" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="AB7" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="AC7" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="AD7" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="AE7" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="AF7" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="AG7" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="AH7" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="AI7" s="8" t="s">
+        <v>243</v>
       </c>
     </row>
-    <row r="5" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>379</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="P5" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="Q5" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="R5" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="S5" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="T5" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="U5" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="V5" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="W5" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="X5" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="Y5" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z5" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="AA5" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="AB5" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="AC5" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="AD5" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="AE5" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="AF5" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="AG5" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="AH5" s="8" t="s">
-        <v>185</v>
+    <row r="8" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="R8" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="S8" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="T8" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="U8" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="AA8" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="AC8" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="AD8" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE8" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="AF8" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="AG8" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="AH8" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="AI8" s="5" t="s">
+        <v>273</v>
       </c>
     </row>
-    <row r="6" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>371</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>380</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="N6" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="O6" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="P6" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="Q6" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="R6" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="S6" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="T6" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="U6" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="V6" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="W6" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="X6" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="Y6" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="Z6" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="AA6" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="AB6" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="AC6" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="AD6" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="AE6" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="AF6" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="AG6" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="AH6" s="8" t="s">
-        <v>214</v>
+    <row r="9" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="L9" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="N9" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="O9" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="P9" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="Q9" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="R9" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="S9" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="T9" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="U9" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="V9" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="W9" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="X9" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="Y9" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="Z9" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="AA9" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="AB9" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="AC9" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="AD9" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="AE9" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="AF9" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="AG9" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="AH9" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="AI9" s="8" t="s">
+        <v>303</v>
       </c>
     </row>
-    <row r="7" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>376</v>
-      </c>
-      <c r="G7" s="6" t="s">
+    <row r="10" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>385</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="N7" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="O7" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="P7" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="Q7" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="R7" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="S7" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="T7" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="U7" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="V7" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="W7" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="X7" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="Y7" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="Z7" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="AA7" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="AB7" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="AC7" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="AD7" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="AE7" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="AF7" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="AG7" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="AH7" s="8" t="s">
-        <v>244</v>
+      <c r="I10" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="N10" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="S10" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="T10" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="U10" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="V10" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="W10" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="X10" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="Y10" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z10" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="AA10" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="AB10" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="AC10" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="AD10" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="AE10" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="AF10" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="AG10" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="AH10" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="AI10" s="5" t="s">
+        <v>334</v>
       </c>
     </row>
-    <row r="8" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>372</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>381</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="M8" s="4" t="s">
-        <v>255</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="O8" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="P8" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="Q8" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="R8" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="S8" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="T8" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="U8" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="V8" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="W8" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="X8" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="Y8" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="Z8" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="AA8" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="AB8" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="AC8" s="4" t="s">
-        <v>269</v>
-      </c>
-      <c r="AD8" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="AE8" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="AF8" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG8" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="AH8" s="8" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="9" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
-        <v>275</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>276</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>278</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="G9" s="6" t="s">
+    <row r="11" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="H11" s="7" t="s">
         <v>382</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>285</v>
-      </c>
-      <c r="N9" s="4" t="s">
-        <v>286</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="P9" s="4" t="s">
-        <v>288</v>
-      </c>
-      <c r="Q9" s="4" t="s">
-        <v>276</v>
-      </c>
-      <c r="R9" s="4" t="s">
-        <v>289</v>
-      </c>
-      <c r="S9" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="T9" s="4" t="s">
-        <v>276</v>
-      </c>
-      <c r="U9" s="4" t="s">
-        <v>291</v>
-      </c>
-      <c r="V9" s="4" t="s">
-        <v>292</v>
-      </c>
-      <c r="W9" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="X9" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="Y9" s="4" t="s">
-        <v>295</v>
-      </c>
-      <c r="Z9" s="4" t="s">
-        <v>296</v>
-      </c>
-      <c r="AA9" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="AB9" s="4" t="s">
-        <v>298</v>
-      </c>
-      <c r="AC9" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="AD9" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="AE9" s="4" t="s">
-        <v>301</v>
-      </c>
-      <c r="AF9" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="AG9" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="AH9" s="8" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="10" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
-        <v>305</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>306</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>309</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>311</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>312</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>313</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>314</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>315</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>316</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="P10" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="Q10" s="4" t="s">
-        <v>319</v>
-      </c>
-      <c r="R10" s="4" t="s">
-        <v>320</v>
-      </c>
-      <c r="S10" s="4" t="s">
-        <v>321</v>
-      </c>
-      <c r="T10" s="4" t="s">
-        <v>306</v>
-      </c>
-      <c r="U10" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="V10" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="W10" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="X10" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="Y10" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="Z10" s="4" t="s">
-        <v>327</v>
-      </c>
-      <c r="AA10" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="AB10" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="AC10" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="AD10" s="4" t="s">
-        <v>331</v>
-      </c>
-      <c r="AE10" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="AF10" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="AG10" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="AH10" s="8" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="11" spans="1:34" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
+      <c r="I11" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="M11" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="N11" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="O11" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="P11" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="Q11" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="R11" s="8" t="s">
         <v>336</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>337</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>338</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>339</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>340</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>375</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>383</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>341</v>
-      </c>
-      <c r="I11" s="10" t="s">
-        <v>342</v>
-      </c>
-      <c r="J11" s="10" t="s">
-        <v>343</v>
-      </c>
-      <c r="K11" s="10" t="s">
-        <v>344</v>
-      </c>
-      <c r="L11" s="10" t="s">
-        <v>345</v>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>346</v>
-      </c>
-      <c r="N11" s="10" t="s">
-        <v>347</v>
-      </c>
-      <c r="O11" s="10" t="s">
-        <v>348</v>
-      </c>
-      <c r="P11" s="10" t="s">
+      <c r="S11" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="Q11" s="10" t="s">
-        <v>337</v>
-      </c>
-      <c r="R11" s="10" t="s">
+      <c r="T11" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="S11" s="10" t="s">
+      <c r="U11" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="V11" s="8" t="s">
         <v>351</v>
       </c>
-      <c r="T11" s="10" t="s">
-        <v>337</v>
-      </c>
-      <c r="U11" s="10" t="s">
+      <c r="W11" s="8" t="s">
         <v>352</v>
       </c>
-      <c r="V11" s="10" t="s">
+      <c r="X11" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="W11" s="10" t="s">
+      <c r="Y11" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="X11" s="10" t="s">
+      <c r="Z11" s="8" t="s">
         <v>355</v>
       </c>
-      <c r="Y11" s="10" t="s">
+      <c r="AA11" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="Z11" s="10" t="s">
+      <c r="AB11" s="8" t="s">
         <v>357</v>
       </c>
-      <c r="AA11" s="10" t="s">
+      <c r="AC11" s="8" t="s">
         <v>358</v>
       </c>
-      <c r="AB11" s="10" t="s">
+      <c r="AD11" s="8" t="s">
         <v>359</v>
       </c>
-      <c r="AC11" s="10" t="s">
+      <c r="AE11" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="AD11" s="10" t="s">
+      <c r="AF11" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="AE11" s="10" t="s">
+      <c r="AG11" s="8" t="s">
         <v>362</v>
       </c>
-      <c r="AF11" s="10" t="s">
+      <c r="AH11" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="AG11" s="10" t="s">
+      <c r="AI11" s="8" t="s">
         <v>364</v>
-      </c>
-      <c r="AH11" s="13" t="s">
-        <v>365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Excel] Update OWASP Top 10 Web 2025
Fix French Threat names
</commit_message>
<xml_diff>
--- a/tools/excel/owasp/owasp-top-10-web_2025.xlsx
+++ b/tools/excel/owasp/owasp-top-10-web_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\owasp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140E4654-EA3E-44CC-8C8A-81CCC0E8CBEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7576D0A9-DAF0-4F00-B213-8E4FFF4B879D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3045" yWindow="-14475" windowWidth="20280" windowHeight="11790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1650" yWindow="-15870" windowWidth="25440" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -84,10 +84,6 @@
   </si>
   <si>
     <t>description[fr]</t>
-  </si>
-  <si>
-    <t>Le Top 10 de l'OWASP est un document de sensibilisation destiné aux développeurs et à la sécurité des applications web. Il représente un large consensus sur les risques de sécurité les plus critiques pour les applications web.
-Source: https://top10.owasp.org/2025/fr/0x00_2025-Introduction/</t>
   </si>
   <si>
     <t>copyright</t>
@@ -1367,9 +1363,6 @@
 For more information about the references and the list of mapped CWEs: https://top10.owasp.org/2025/A03_2025-Software_Supply_Chain_Failures/</t>
   </si>
   <si>
-    <t>Défaillances de la nomenclature logicielle</t>
-  </si>
-  <si>
     <t>Selhání dodavatelského řetězce softwaru (Software Supply Chain Failures)</t>
   </si>
   <si>
@@ -5316,9 +5309,6 @@
 For more information about the references and the list of mapped CWEs: https://top10.owasp.org/2025/A08_2025-Software_or_Data_Integrity_Failures/</t>
   </si>
   <si>
-    <t>Manque d'intégrité des données ou du logiciel</t>
-  </si>
-  <si>
     <t>Selhání integrity softwaru nebo dat (Software or Data Integrity Failures)</t>
   </si>
   <si>
@@ -5905,9 +5895,6 @@
 **Scenario #2:** A major Indian airline had a data breach involving more than ten years' worth of personal data of millions of passengers, including passport and credit card data. The data breach occurred at a third-party cloud hosting provider, who notified the airline of the breach after some time.
 **Scenario #3:** A major European airline suffered a GDPR reportable breach. The breach was reportedly caused by payment application security vulnerabilities exploited by attackers, who harvested more than 400,000 customer payment records. The airline was fined 20 million pounds as a result by the privacy regulator.
 For more information about the references and the list of mapped CWEs: https://top10.owasp.org/2025/A09_2025-Security_Logging_and_Alerting_Failures/</t>
-  </si>
-  <si>
-    <t>Carence des systèmes de contrôle et d'alerte</t>
   </si>
   <si>
     <t>Selhání bezpečnostního logování a upozorňování (Security Logging &amp; Alerting Failures)</t>
@@ -6488,9 +6475,6 @@
 Exceptional conditions can be caused by missing, poor, or incomplete input validation, or late, high level error handling instead at the functions where they occur, or unexpected environmental states such as memory, privilege, or network issues, inconsistent exception handling, or exceptions that are not handled at all, allowing the system to fall into an unknown and unpredictable state. Any time an application is unsure of its next instruction, an exceptional condition has been mishandled. Hard-to-find errors and exceptions can threaten the security of the whole application for a long time.
 Many different security vulnerabilities can happen when we mishandle exceptional conditions,
 such as logic bugs, overflows, race conditions, fraudulent transactions, or issues with memory, state, resource, timing, authentication, and authorization. These types of vulnerabilities can negatively affect the confidentiality, availability, and/or integrity of a system or it’s data. Attackers manipulate an application's flawed error handling to strike this vulnerability. </t>
-  </si>
-  <si>
-    <t>Mauvaise gestion des exceptions</t>
   </si>
   <si>
     <t>Nesprávné zpracování výjimečných stavů (Mishandling of Exceptional Conditions)</t>
@@ -8650,6 +8634,22 @@
 **Scénario #3 :** La corruption d’état dans les transactions financières pourrait être causée par un attaquant interrompant une transaction en plusieurs étapes via des perturbations réseau. Imaginez que l’ordre de la transaction soit : débiter un compte utilisateur, créditer le compte de destination, enregistrer la transaction. Si le système ne revient pas correctement sur l’intégralité de la transaction (échec fermé) en cas d’erreur en cours de route, l’attaquant pourrait potentiellement vider le compte de l’utilisateur, ou peut-être une condition de course permettant à l’attaquant d’envoyer de l’argent à destination plusieurs fois. 
 Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A10_2025-Mishandling_of_Exceptional_Conditions/</t>
   </si>
+  <si>
+    <t>Défaillances de la chaîne d’approvisionnement logicielle</t>
+  </si>
+  <si>
+    <t>Défaillances de la journalisation et de l'alerte de sécurité</t>
+  </si>
+  <si>
+    <t>Mauvaise gestion des conditions exceptionnelles</t>
+  </si>
+  <si>
+    <t>Défaillances logicielles ou d'intégrité des données</t>
+  </si>
+  <si>
+    <t>Le Top 10 de l'OWASP est un document de sensibilisation destiné aux développeurs et à la sécurité des applications web. Il représente un large consensus sur les risques de sécurité les plus critiques pour les applications web.
+Source: https://top10.owasp.org/2025/0x00_2025-Introduction/</t>
+  </si>
 </sst>
 </file>
 
@@ -8678,7 +8678,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -8700,6 +8700,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor theme="0" tint="-0.14999847407452621"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor theme="0" tint="-0.14999847407452621"/>
       </patternFill>
     </fill>
@@ -8771,7 +8777,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -8802,6 +8808,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10366,7 +10378,7 @@
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="3" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -10426,40 +10438,40 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>16</v>
+      <c r="B9" s="14" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>11</v>
@@ -10467,15 +10479,15 @@
     </row>
     <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>11</v>
@@ -10483,15 +10495,15 @@
     </row>
     <row r="16" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>11</v>
@@ -10499,15 +10511,15 @@
     </row>
     <row r="18" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>11</v>
@@ -10515,15 +10527,15 @@
     </row>
     <row r="20" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>11</v>
@@ -10531,15 +10543,15 @@
     </row>
     <row r="22" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>11</v>
@@ -10547,15 +10559,15 @@
     </row>
     <row r="24" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>11</v>
@@ -10563,15 +10575,15 @@
     </row>
     <row r="26" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>11</v>
@@ -10579,15 +10591,15 @@
     </row>
     <row r="28" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>11</v>
@@ -10595,10 +10607,10 @@
     </row>
     <row r="30" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -10620,15 +10632,15 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -10683,7 +10695,7 @@
         <v>8</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>10</v>
@@ -10692,7 +10704,7 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F1" s="12" t="s">
         <v>14</v>
@@ -10701,1158 +10713,1158 @@
         <v>15</v>
       </c>
       <c r="H1" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="I1" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="K1" s="12" t="s">
+      <c r="L1" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M1" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="N1" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="L1" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="M1" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="12" t="s">
+      <c r="O1" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="P1" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q1" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="O1" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="P1" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q1" s="12" t="s">
+      <c r="R1" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="S1" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="T1" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="R1" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="S1" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="T1" s="12" t="s">
+      <c r="U1" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="V1" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="W1" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="U1" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="V1" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="W1" s="12" t="s">
+      <c r="X1" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y1" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z1" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="X1" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="Y1" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z1" s="12" t="s">
+      <c r="AA1" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB1" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC1" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="AA1" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="AB1" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC1" s="12" t="s">
+      <c r="AD1" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="AE1" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF1" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="AD1" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="AE1" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="AF1" s="12" t="s">
+      <c r="AG1" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="AI1" s="12" t="s">
         <v>61</v>
-      </c>
-      <c r="AG1" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="AH1" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI1" s="12" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="I2" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="G2" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>346</v>
-      </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="R2" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="T2" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="U2" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="V2" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="U2" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="V2" s="5" t="s">
+      <c r="W2" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="W2" s="5" t="s">
+      <c r="X2" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="X2" s="5" t="s">
+      <c r="Y2" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="Y2" s="5" t="s">
+      <c r="Z2" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="Z2" s="5" t="s">
+      <c r="AA2" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="AA2" s="5" t="s">
+      <c r="AB2" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="AB2" s="5" t="s">
+      <c r="AC2" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="AC2" s="5" t="s">
+      <c r="AD2" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="AD2" s="5" t="s">
+      <c r="AE2" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AE2" s="5" t="s">
+      <c r="AF2" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="AF2" s="5" t="s">
+      <c r="AG2" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="AG2" s="5" t="s">
+      <c r="AH2" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="AH2" s="5" t="s">
+      <c r="AI2" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="AI2" s="5" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>352</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>357</v>
-      </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="G3" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="N3" s="8" t="s">
         <v>366</v>
       </c>
-      <c r="F3" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>395</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="K3" s="8" t="s">
+      <c r="O3" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="P3" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q3" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="R3" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="S3" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="T3" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="U3" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="V3" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="W3" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="X3" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Y3" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z3" s="8" t="s">
         <v>369</v>
       </c>
-      <c r="L3" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="M3" s="8" t="s">
+      <c r="AA3" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="AB3" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="AC3" s="8" t="s">
         <v>370</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="AD3" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="AE3" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF3" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="O3" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="P3" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="Q3" s="8" t="s">
+      <c r="AG3" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="AH3" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="AI3" s="8" t="s">
         <v>372</v>
-      </c>
-      <c r="R3" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="S3" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="T3" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="U3" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="V3" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="W3" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="X3" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="Y3" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="Z3" s="8" t="s">
-        <v>374</v>
-      </c>
-      <c r="AA3" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="AB3" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="AC3" s="8" t="s">
-        <v>375</v>
-      </c>
-      <c r="AD3" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="AE3" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="AF3" s="8" t="s">
-        <v>376</v>
-      </c>
-      <c r="AG3" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="AH3" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="AI3" s="8" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="4" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G4" s="6" t="s">
-        <v>339</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>351</v>
-      </c>
-      <c r="I4" s="5" t="s">
+      <c r="K4" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="L4" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="M4" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="N4" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="O4" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="P4" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="Q4" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="P4" s="5" t="s">
+      <c r="R4" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="Q4" s="5" t="s">
+      <c r="S4" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="R4" s="5" t="s">
+      <c r="T4" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="S4" s="5" t="s">
+      <c r="U4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="V4" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="T4" s="5" t="s">
+      <c r="W4" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="U4" s="5" t="s">
+      <c r="X4" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AB4" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="V4" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="W4" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="X4" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="Y4" s="5" t="s">
+      <c r="AC4" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="Z4" s="5" t="s">
+      <c r="AD4" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="AA4" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB4" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="AC4" s="5" t="s">
+      <c r="AE4" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="AD4" s="5" t="s">
+      <c r="AF4" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="AE4" s="5" t="s">
+      <c r="AG4" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="AF4" s="5" t="s">
+      <c r="AH4" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="AG4" s="5" t="s">
+      <c r="AI4" s="5" t="s">
         <v>141</v>
-      </c>
-      <c r="AH4" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="AI4" s="5" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="5" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>359</v>
-      </c>
-      <c r="C5" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="G5" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>340</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>347</v>
-      </c>
-      <c r="I5" s="8" t="s">
+      <c r="K5" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="M5" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="N5" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="M5" s="8" t="s">
+      <c r="O5" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="N5" s="8" t="s">
+      <c r="P5" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="O5" s="8" t="s">
+      <c r="Q5" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="P5" s="8" t="s">
+      <c r="R5" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="Q5" s="8" t="s">
+      <c r="S5" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="R5" s="8" t="s">
+      <c r="T5" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="S5" s="8" t="s">
+      <c r="U5" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="V5" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="T5" s="8" t="s">
+      <c r="W5" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="U5" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="V5" s="8" t="s">
+      <c r="X5" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="W5" s="8" t="s">
+      <c r="Y5" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="X5" s="8" t="s">
+      <c r="Z5" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="Y5" s="8" t="s">
+      <c r="AA5" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="Z5" s="8" t="s">
+      <c r="AB5" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="AA5" s="8" t="s">
+      <c r="AC5" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AB5" s="8" t="s">
+      <c r="AD5" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="AC5" s="8" t="s">
+      <c r="AE5" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="AD5" s="8" t="s">
+      <c r="AF5" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="AE5" s="8" t="s">
+      <c r="AG5" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="AF5" s="8" t="s">
+      <c r="AH5" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="AG5" s="8" t="s">
+      <c r="AI5" s="8" t="s">
         <v>172</v>
-      </c>
-      <c r="AH5" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="AI5" s="8" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>360</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="F6" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="J6" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>341</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>348</v>
-      </c>
-      <c r="I6" s="5" t="s">
+      <c r="K6" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="L6" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="M6" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="N6" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="L6" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="M6" s="5" t="s">
+      <c r="O6" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="P6" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="O6" s="5" t="s">
+      <c r="Q6" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="P6" s="5" t="s">
+      <c r="R6" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="Q6" s="5" t="s">
+      <c r="S6" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="R6" s="5" t="s">
+      <c r="T6" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="S6" s="5" t="s">
+      <c r="U6" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="V6" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="T6" s="5" t="s">
+      <c r="W6" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="U6" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="V6" s="5" t="s">
+      <c r="X6" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="W6" s="5" t="s">
+      <c r="Y6" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="X6" s="5" t="s">
+      <c r="Z6" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="Y6" s="5" t="s">
+      <c r="AA6" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="Z6" s="5" t="s">
+      <c r="AB6" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="AA6" s="5" t="s">
+      <c r="AC6" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="AB6" s="5" t="s">
+      <c r="AD6" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="AC6" s="5" t="s">
+      <c r="AE6" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="AD6" s="5" t="s">
+      <c r="AF6" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="AE6" s="5" t="s">
+      <c r="AG6" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="AF6" s="5" t="s">
+      <c r="AH6" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="AG6" s="5" t="s">
+      <c r="AI6" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="AH6" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="AI6" s="5" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>361</v>
-      </c>
-      <c r="C7" s="8" t="s">
+      <c r="E7" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="G7" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="I7" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="G7" s="6" t="s">
-        <v>345</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="I7" s="8" t="s">
+      <c r="K7" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="M7" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="L7" s="8" t="s">
+      <c r="N7" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="M7" s="8" t="s">
+      <c r="O7" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="N7" s="8" t="s">
+      <c r="P7" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="O7" s="8" t="s">
+      <c r="Q7" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="P7" s="8" t="s">
+      <c r="R7" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="S7" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="Q7" s="8" t="s">
+      <c r="T7" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="R7" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="S7" s="8" t="s">
+      <c r="U7" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="V7" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="T7" s="8" t="s">
+      <c r="W7" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="U7" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="V7" s="8" t="s">
+      <c r="X7" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="W7" s="8" t="s">
+      <c r="Y7" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="X7" s="8" t="s">
+      <c r="Z7" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="Y7" s="8" t="s">
+      <c r="AA7" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="Z7" s="8" t="s">
+      <c r="AB7" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="AA7" s="8" t="s">
+      <c r="AC7" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="AB7" s="8" t="s">
+      <c r="AD7" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="AC7" s="8" t="s">
+      <c r="AE7" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="AD7" s="8" t="s">
+      <c r="AF7" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="AE7" s="8" t="s">
+      <c r="AG7" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="AF7" s="8" t="s">
+      <c r="AH7" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="AG7" s="8" t="s">
+      <c r="AI7" s="8" t="s">
         <v>231</v>
-      </c>
-      <c r="AH7" s="8" t="s">
-        <v>232</v>
-      </c>
-      <c r="AI7" s="8" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="8" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="G8" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="I8" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="J8" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>342</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>349</v>
-      </c>
-      <c r="I8" s="5" t="s">
+      <c r="K8" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="L8" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="M8" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="N8" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="M8" s="5" t="s">
+      <c r="O8" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="N8" s="5" t="s">
+      <c r="P8" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="O8" s="5" t="s">
+      <c r="Q8" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="P8" s="5" t="s">
+      <c r="R8" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="S8" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="Q8" s="5" t="s">
+      <c r="T8" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="R8" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="S8" s="5" t="s">
+      <c r="U8" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="V8" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="T8" s="5" t="s">
+      <c r="W8" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="U8" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="V8" s="5" t="s">
+      <c r="X8" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="W8" s="5" t="s">
+      <c r="Y8" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="Z8" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="X8" s="5" t="s">
+      <c r="AA8" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="Y8" s="5" t="s">
-        <v>378</v>
-      </c>
-      <c r="Z8" s="5" t="s">
+      <c r="AB8" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="AA8" s="5" t="s">
+      <c r="AC8" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="AB8" s="5" t="s">
+      <c r="AD8" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="AC8" s="5" t="s">
+      <c r="AE8" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="AD8" s="5" t="s">
+      <c r="AF8" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="AE8" s="5" t="s">
+      <c r="AG8" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="AF8" s="5" t="s">
+      <c r="AH8" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="AG8" s="5" t="s">
+      <c r="AI8" s="5" t="s">
         <v>260</v>
-      </c>
-      <c r="AH8" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="AI8" s="5" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="9" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>363</v>
-      </c>
-      <c r="C9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="F9" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="J9" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="K9" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>343</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>350</v>
-      </c>
-      <c r="I9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="M9" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="N9" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="O9" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="P9" s="8" t="s">
         <v>272</v>
       </c>
-      <c r="N9" s="8" t="s">
+      <c r="Q9" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="O9" s="8" t="s">
+      <c r="R9" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="S9" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="P9" s="8" t="s">
+      <c r="T9" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="Q9" s="8" t="s">
+      <c r="U9" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="V9" s="8" t="s">
         <v>276</v>
       </c>
-      <c r="R9" s="8" t="s">
-        <v>264</v>
-      </c>
-      <c r="S9" s="8" t="s">
+      <c r="W9" s="8" t="s">
         <v>277</v>
       </c>
-      <c r="T9" s="8" t="s">
+      <c r="X9" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="U9" s="8" t="s">
-        <v>264</v>
-      </c>
-      <c r="V9" s="8" t="s">
+      <c r="Y9" s="8" t="s">
         <v>279</v>
       </c>
-      <c r="W9" s="8" t="s">
+      <c r="Z9" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="X9" s="8" t="s">
+      <c r="AA9" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="Y9" s="8" t="s">
+      <c r="AB9" s="8" t="s">
         <v>282</v>
       </c>
-      <c r="Z9" s="8" t="s">
+      <c r="AC9" s="8" t="s">
         <v>283</v>
       </c>
-      <c r="AA9" s="8" t="s">
+      <c r="AD9" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="AB9" s="8" t="s">
+      <c r="AE9" s="8" t="s">
         <v>285</v>
       </c>
-      <c r="AC9" s="8" t="s">
+      <c r="AF9" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="AD9" s="8" t="s">
+      <c r="AG9" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="AE9" s="8" t="s">
+      <c r="AH9" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="AF9" s="8" t="s">
+      <c r="AI9" s="8" t="s">
         <v>289</v>
-      </c>
-      <c r="AG9" s="8" t="s">
-        <v>290</v>
-      </c>
-      <c r="AH9" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="AI9" s="8" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="10" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>394</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>364</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="J10" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="K10" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>367</v>
-      </c>
-      <c r="E10" s="5" t="s">
+      <c r="L10" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="M10" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="N10" s="5" t="s">
         <v>296</v>
       </c>
-      <c r="G10" s="6" t="s">
-        <v>396</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>353</v>
-      </c>
-      <c r="I10" s="5" t="s">
+      <c r="O10" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="P10" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="S10" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="T10" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="U10" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="V10" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="W10" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="X10" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="Y10" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="Z10" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="AA10" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="AB10" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="K10" s="5" t="s">
-        <v>298</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="M10" s="5" t="s">
+      <c r="AC10" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="AD10" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="AE10" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="N10" s="5" t="s">
-        <v>300</v>
-      </c>
-      <c r="O10" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="P10" s="5" t="s">
+      <c r="AF10" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="AG10" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="AH10" s="5" t="s">
         <v>381</v>
       </c>
-      <c r="Q10" s="5" t="s">
-        <v>302</v>
-      </c>
-      <c r="R10" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="S10" s="5" t="s">
-        <v>304</v>
-      </c>
-      <c r="T10" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="U10" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="V10" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="W10" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="X10" s="5" t="s">
-        <v>307</v>
-      </c>
-      <c r="Y10" s="5" t="s">
-        <v>383</v>
-      </c>
-      <c r="Z10" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="AA10" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="AB10" s="5" t="s">
-        <v>384</v>
-      </c>
-      <c r="AC10" s="5" t="s">
+      <c r="AI10" s="5" t="s">
         <v>310</v>
-      </c>
-      <c r="AD10" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="AE10" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="AF10" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="AG10" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="AH10" s="5" t="s">
-        <v>386</v>
-      </c>
-      <c r="AI10" s="5" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="11" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="J11" s="8" t="s">
         <v>315</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>365</v>
-      </c>
-      <c r="C11" s="8" t="s">
+      <c r="K11" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="L11" s="8" t="s">
         <v>316</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="M11" s="8" t="s">
         <v>317</v>
       </c>
-      <c r="E11" s="8" t="s">
-        <v>368</v>
-      </c>
-      <c r="F11" s="8" t="s">
+      <c r="N11" s="8" t="s">
+        <v>383</v>
+      </c>
+      <c r="O11" s="8" t="s">
         <v>318</v>
       </c>
-      <c r="G11" s="6" t="s">
-        <v>344</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>397</v>
-      </c>
-      <c r="I11" s="8" t="s">
+      <c r="P11" s="8" t="s">
         <v>319</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="Q11" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="R11" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="S11" s="8" t="s">
         <v>320</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="T11" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="U11" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="V11" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="W11" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="X11" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="Y11" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z11" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="AA11" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="AB11" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="AC11" s="8" t="s">
         <v>387</v>
       </c>
-      <c r="L11" s="8" t="s">
-        <v>321</v>
-      </c>
-      <c r="M11" s="8" t="s">
-        <v>322</v>
-      </c>
-      <c r="N11" s="8" t="s">
+      <c r="AD11" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="AE11" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="AF11" s="8" t="s">
         <v>388</v>
       </c>
-      <c r="O11" s="8" t="s">
-        <v>323</v>
-      </c>
-      <c r="P11" s="8" t="s">
-        <v>324</v>
-      </c>
-      <c r="Q11" s="8" t="s">
+      <c r="AG11" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="AH11" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="AI11" s="8" t="s">
         <v>389</v>
-      </c>
-      <c r="R11" s="8" t="s">
-        <v>316</v>
-      </c>
-      <c r="S11" s="8" t="s">
-        <v>325</v>
-      </c>
-      <c r="T11" s="8" t="s">
-        <v>326</v>
-      </c>
-      <c r="U11" s="8" t="s">
-        <v>316</v>
-      </c>
-      <c r="V11" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="W11" s="8" t="s">
-        <v>390</v>
-      </c>
-      <c r="X11" s="8" t="s">
-        <v>328</v>
-      </c>
-      <c r="Y11" s="8" t="s">
-        <v>329</v>
-      </c>
-      <c r="Z11" s="8" t="s">
-        <v>391</v>
-      </c>
-      <c r="AA11" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="AB11" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="AC11" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="AD11" s="8" t="s">
-        <v>332</v>
-      </c>
-      <c r="AE11" s="8" t="s">
-        <v>333</v>
-      </c>
-      <c r="AF11" s="8" t="s">
-        <v>393</v>
-      </c>
-      <c r="AG11" s="8" t="s">
-        <v>334</v>
-      </c>
-      <c r="AH11" s="8" t="s">
-        <v>335</v>
-      </c>
-      <c r="AI11" s="8" t="s">
-        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[YAML & Excel] Update OWASP Top 10 Web 2025
Minor fixes in French Link and [fa] code block
</commit_message>
<xml_diff>
--- a/tools/excel/owasp/owasp-top-10-web_2025.xlsx
+++ b/tools/excel/owasp/owasp-top-10-web_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\owasp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294CA6D2-75F6-4A1C-BA8F-D6C3D42439A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{284B60DC-2255-4389-A01C-20E826156023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1650" yWindow="-15870" windowWidth="25440" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1650" yWindow="-15870" windowWidth="25440" windowHeight="15990" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -2509,69 +2509,6 @@
    &lt;/td&gt;
   &lt;/tr&gt;
   &lt;tr&gt;
-   &lt;td&gt;36
-   &lt;/td&gt;
-   &lt;td&gt;15,80 % 
-   &lt;/td&gt;
-   &lt;td&gt;2,92 % 
-   &lt;/td&gt;
-   &lt;td&gt;100,00 % 
-   &lt;/td&gt;
-   &lt;td&gt;37,14 % 
-   &lt;/td&gt;
-   &lt;td&gt;7,69
-   &lt;/td&gt;
-   &lt;td&gt;4,44
-   &lt;/td&gt;
-   &lt;td&gt;1 120 673
-   &lt;/td&gt;
-   &lt;td&gt;7 147
-   &lt;/td&gt;
-  &lt;/tr&gt;
-&lt;/table&gt;
-## Comment prévenir
-* Lorsque possible, implémenter et faire respecter l’utilisation de l’authentification multifactorielle pour prévenir le bourrage automatisé des identifiants, la force brute et les attaques de réutilisation de crédents volées. 
-* Lorsque possible, encourager et activer l’utilisation de gestionnaires de mots de passe pour aider les utilisateurs à faire de meilleurs choix. 
-* Ne pas livrer ni déployer avec des identifiants par défaut, en particulier pour les utilisateurs administrateurs. 
-* Mettre en place des vérifications de mots de passe faibles, comme tester de nouveaux mots de passe ou modifiés dans la liste des 10 000 pires mots de passe. 
-* Lors de la création d’un nouveau compte et des changements de mot de passe, validez contre les listes d’identifiants connus pour violation (par exemple : utiliser [haveibeenpwned.com](https://haveibeenpwned.com)). 
-* Aligner les politiques de longueur, de complexité et de rotation des mots de passe avec les directives du [National Institute of Standards and Technology (NIST) 800-63b dans la section 5.1.1] (https://pages.nist.gov/800-63-3/sp800-63b.html#:~:text=5.1.1%20Memorized%20Secrets) pour les secrets mémorisés ou d’autres politiques modernes fondées sur des mots de passe fondées sur des preuves. 
-* Ne forcez pas les êtres humains à faire tourner les mots de passe sauf si vous suspectez une faille. Si vous soupçonnez une fuite, forcez immédiatement la réinitialisation du mot de passe.  
-* S’assurer que l’enregistrement, la récupération des identifiants et les voies API sont renforcés contre les attaques d’énumération de comptes en utilisant les mêmes messages pour tous les résultats (« Nom d’utilisateur ou mot de passe invalides. »). 
-* Limiter ou retarder de plus en plus les tentatives de connexion ratées, mais veillez à ne pas créer un scénario de déni de service. Consignez toutes les défaillances et alertez les administrateurs lorsque des attaques de type « credentialsal stuffing, de force brute » ou d’autres attaques sont détectées ou suspectées. 
-* Utiliser un gestionnaire de session intégré sécurisé côté serveur qui génère un nouvel ID de session aléatoire avec une forte entropie après la connexion. Les identifiants de session ne doivent pas être dans l’URL, être stockés de manière sécurisée dans un cookie sécurisé, et invalidés après déconnexion, inactivité et délais absolus.  
-* Idéalement, utiliser un système préfabriqué et bien fiable pour gérer l’authentification, l’identité et la gestion des sessions. Transférez ce risque autant que possible en achetant et en utilisant un système renforcé et bien testé. 
-* Vérifier l’utilisation prévue des identifiants fournis, par exemple pour les JWT, valider les affirmations « aud », « iss » et les périmètres
-## Exemples de scénarios d’attaque
-**Scénario #1 :** Le remplissage de crédentiaux, l’utilisation de listes de combinaisons de noms d’utilisateur et de mots de passe connus, est désormais une attaque très courante. Plus récemment, les attaquants ont été observés « incrémentant » ou ajustant autrement les mots de passe, en fonction du comportement humain courant. Par exemple, changer « Winter2025 » en « Hiver 2026 », ou « ILoveMyDog6 » en « ILoveMyDog7 » ou « ILoveMyDog5 ». Cet ajustement des tentatives de mot de passe est appelé attaque hybride de remplissage de crédibles ou attaque par pulvérisation de mots de passe, et ils peuvent être encore plus efficaces que la version traditionnelle. Si une application ne met pas en place de défenses contre les menaces automatisées (force brute, scripts ou bots) ou bourrage de crédents, l’application peut être utilisée comme oracle de mot de passe pour déterminer si les identifiants sont valides et obtenir un accès non autorisé. 
-**Scénario #2 :** La plupart des attaques d’authentification réussies surviennent en raison de l’utilisation continue des mots de passe comme seul facteur d’authentification. Une fois considérées comme les meilleures pratiques, la rotation des mots de passe et les exigences de complexité encouragent les utilisateurs à réutiliser les mots de passe et à utiliser des mots de passe faibles. Il est recommandé aux organisations d’arrêter ces pratiques conformément au NIST 800-63 et d’imposer l’utilisation de l’authentification multifacteur sur tous les systèmes importants. 
-**Scénario #3 :** Les délais d’expiration des sessions d’application ne sont pas correctement implémentés. Un utilisateur utilise un ordinateur public pour accéder à une application et au lieu de sélectionner « déconnexion », il ferme simplement l’onglet du navigateur et s’en va. Un autre exemple est si une session de connexion unique (SSO) ne peut pas être fermée par un seul déconnexion (SLO). C’est-à-dire qu’une seule connexion vous connecte, par exemple, à votre lecteur de messagerie, à votre système de documents et à votre système de chat. Mais la déconnexion ne se produit qu’au système actuel. Si un attaquant utilise le même navigateur après que la victime pense s’être déconnectée avec succès, mais avec l’utilisateur toujours authentifié sur certaines applications, il peut alors accéder au compte de la victime. Le même problème peut survenir dans les bureaux et les entreprises lorsqu’une application sensible n’a pas été correctement fermée et qu’un collègue a un accès (temporaire) à l’ordinateur déverrouillé. 
-Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A07_2025-Authentication_Failures/</t>
-  </si>
-  <si>
-    <t>## Tableau des scores
-&lt;table&gt;
-  &lt;tr&gt;
-   &lt;td&gt;CWEs cartographiées 
-   &lt;/td&gt;
-   &lt;td&gt;Taux d’incidence maximal
-   &lt;/td&gt;
-   &lt;td&gt;Taux moyen d’incidence
-   &lt;/td&gt;
-   &lt;td&gt;Couverture maximale
-   &lt;/td&gt;
-   &lt;td&gt;Couverture moyenne
-   &lt;/td&gt;
-   &lt;td&gt;Exploit pondéré moyen
-   &lt;/td&gt;
-   &lt;td&gt;Impact pondéré moyen
-   &lt;/td&gt;
-   &lt;td&gt;Occurrences totales
-   &lt;/td&gt;
-   &lt;td&gt;Total des CVE
-   &lt;/td&gt;
-  &lt;/tr&gt;
-  &lt;tr&gt;
    &lt;td&gt;14
    &lt;/td&gt;
    &lt;td&gt;8,98 % 
@@ -2604,90 +2541,6 @@
 **Scénario #3 Utilisation d’un paquet à partir d’une source non fiable :** Un développeur a du mal à trouver la version mise à jour d’un paquet qu’il recherche, il la télécharge donc non pas depuis le gestionnaire de paquets fiable classique, mais depuis un site web en ligne. Le paquet n’est pas signé, et il n’y a donc aucune possibilité d’en garantir l’intégrité. Le paquet inclut du code malveillant. 
 **Scénario #4 Désérialisation insécurisée :** Une application React appelle un ensemble de microservices Spring Boot. En tant que programmeurs fonctionnels, ils ont essayé de s’assurer que leur code reste immuable. La solution qu’ils ont trouvée est de sérialiser l’état utilisateur et de le transmettre à chaque requête. Un attaquant remarque la signature d’objet Java « rO0 » (en base64) et utilise le [Java Deserialization Scanner](https://github.com/federicodotta/Java-Deserialization-Scanner) pour obtenir une exécution de code à distance sur le serveur d’applications. 
 Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A08_2025-Software_or_Data_Integrity_Failures/</t>
-  </si>
-  <si>
-    <t>## Tableau des scores
-&lt;table&gt;
-  &lt;tr&gt;
-   &lt;td&gt;CWEs cartographiées
-   &lt;/td&gt;
-   &lt;td&gt;Taux d’incidence maximal
-   &lt;/td&gt;
-   &lt;td&gt;Taux moyen d’incidence
-   &lt;/td&gt;
-   &lt;td&gt;Couverture maximale
-   &lt;/td&gt;
-   &lt;td&gt;Couverture moyenne
-   &lt;/td&gt;
-   &lt;td&gt;Exploit pondéré moyen
-   &lt;/td&gt;
-   &lt;td&gt;Impact pondéré moyen
-   &lt;/td&gt;
-   &lt;td&gt;Occurrences totales
-   &lt;/td&gt;
-   &lt;td&gt;Total des CVE
-   &lt;/td&gt;
-  &lt;/tr&gt;
-  &lt;tr&gt;
-   &lt;td&gt;6
-   &lt;/td&gt;
-   &lt;td&gt;9,56 % 
-   &lt;/td&gt;
-   &lt;td&gt;5,72 % 
-   &lt;/td&gt;
-   &lt;td&gt;65,42 % 
-   &lt;/td&gt;
-   &lt;td&gt;27,47 % 
-   &lt;/td&gt;
-   &lt;td&gt;8.17
-   &lt;/td&gt;
-   &lt;td&gt;5.23
-   &lt;/td&gt;
-   &lt;td&gt;215 248
-   &lt;/td&gt;
-   &lt;td&gt;11
-   &lt;/td&gt;
-  &lt;/tr&gt;
-&lt;/table&gt;
-## Comment prévenir
-Il devrait y avoir un processus de gestion des correctifs pour : 
-* Générer et gérer centralisément la liste des documents logiciels (SBOM) de l’ensemble de votre logiciel. 
-* Suivre non seulement vos dépendances directes, mais aussi leurs dépendances (transitives), et ainsi de suite. 
-* Réduire la surface d’attaque en supprimant les dépendances inutilisées, les fonctionnalités, les composants, les fichiers et la documentation inutiles. 
-* Inventorier continuellement les versions des composants côté client et côté serveur (par exemple, frameworks, bibliothèques) et leurs dépendances à l’aide d’outils comme OWASP Dependency Track, OWASP Dependency Check, retire.js, etc. 
-* Surveillez en continu des sources telles que Common Vulnerability and Exposures (CVE), National Vulnerability Database (NVD) et [Open Source Vulnerabilities (OSV)](https://osv.dev/) pour les vulnérabilités des composants que vous utilisez. Utilisez l’analyse de composition logicielle, la chaîne d’approvisionnement logicielle ou des outils SBOM axés sur la sécurité pour automatiser le processus. Abonnez-vous aux alertes concernant les vulnérabilités de sécurité liées aux composants que vous utilisez. 
-* N’obtenir les composants que de sources officielles (fiables) via des liens sécurisés. Privilégier les paquets signés pour réduire le risque d’inclure un composant modifié et malveillant (voir [A08:2025 - Défaillances d’intégrité logicielle et des données](https://owasp.org/Top10/2025/A08_2025-Software_or_Data_Integrity_Failures/)). 
-* Choisissez délibérément la version d’une dépendance que vous utilisez et ne mettez à jour que lorsqu’il y a un besoin. 
-* Surveillez les bibliothèques et composants non maintenus ou qui ne créent pas de correctifs de sécurité pour les versions précédentes. Si le patch n’est pas possible, envisagez de migrer vers une alternative. Si cela n’est pas possible, envisagez de déployer un correctif virtuel pour surveiller, détecter ou protéger contre le problème découvert. 
-* Mettez régulièrement à jour votre CI/CD, IDE et tout autre outil de développement
-* Éviter de déployer des mises à jour simultanément sur tous les systèmes. Utiliser des déploiements par étapes ou des déploiements canari pour limiter l’exposition au cas où un fournisseur de confiance serait compromis. 
-Il devrait y avoir un processus de gestion des changements ou un système de suivi pour suivre les modifications sur :
-* Paramètres CI/CD (tous les outils de compilation et pipelines)
-* Dépôts de code
-* Zones de bac à sable
-* IDE développeurs
-* Outils SBOM et artefacts créés
-* Systèmes de journalisation et journaux
-* Intégrations tierces, telles que le SaaS
-* Dépôts d’artefacts
-* Registres de conteneurs
-Renforcez les systèmes suivants, ce qui inclut la mise en service de la MFA et la fermeture de l’IAM : 
-* Votre dépôt de code (ce qui inclut de ne pas vérifier les secrets, protéger les branches, sauvegarder)
-* Stations de travail développeurs (correctifs réguliers, MFA, surveillance, et plus encore)
-* Votre serveur de compilation &amp; CI/CD (séparation des fonctions, contrôle d’accès, compilations signées, secrets à portée d’environnement, journaux inviolables, plus encore)
-* Vos artefacts (assurez l’intégrité via la provenance, la signature et l’horodatage, promouvez les artefacts plutôt que les reconstruisez pour chaque environnement, assurez-vous que les builds restent immuables)
-* Infrastructure en tant que code (géré comme tout le code, y compris l’utilisation des PR et le contrôle de versions)
-Chaque organisation doit s’assurer d’un plan continu pour la surveillance, le tri et l’application des mises à jour ou modifications de configuration tout au long de la durée de vie de l’application ou du portefeuille.
-## Exemples de scénarios d’attaque
-**Scénario #1 :** Un fournisseur de confiance est compromis par des logiciels malveillants, ce qui entraîne la compromission de vos systèmes informatiques lors de la mise à jour. L’exemple le plus célèbre est probablement : 
-* Le compromis SolarWinds de 2019 qui a conduit à la compromission de ~18 000 organisations. [https://www.npr.org/2021/04/16/985439655/a-worst-nightmare-cyberattack-the-untold-story-of-the-solarwinds-hack] (https://www.npr.org/2021/04/16/985439655/a-worst-nightmare-cyberattack-the-untold-story-of-the-solarwinds-hack)
-**Scénario #2 :** Un fournisseur de confiance est compromis au point de ne se comporter de manière malveillante que dans une condition spécifique. 
-* Le vol de 1,5 milliard de dollars par Bybit en 2025 a été causé par [une attaque de chaîne d’approvisionnement dans un logiciel de portefeuille](https://www.sygnia.co/blog/sygnia-investigation-bybit-hack/) qui ne s’est exécutée que lorsque le portefeuille cible était utilisé. 
-**Scénario #3 :** L’attaque de chaîne d’approvisionnement ['Shai-Hulud'](https://www.cisa.gov/news-events/alerts/2025/09/23/widespread-supply-chain-compromise-impacting-npm-ecosystem) en 2025 a été le premier ver npm auto-propagant réussi. Les attaques ont semé des versions malveillantes de paquets populaires, qui utilisaient un script post-installation pour récolter et exfiltrer des données sensibles vers des dépôts publics GitHub. Le malware détectait également les jetons npm dans l’environnement victime et les utilisait automatiquement pour diffuser des versions malveillantes de tout package accessible. Le ver a atteint plus de 500 versions de paquets avant d’être perturbé par npm. Cette attaque de chaîne d’approvisionnement était avancée, se propageait rapidement et causait des dommages, et en ciblant les machines développeurs, elle a démontré que les développeurs eux-mêmes sont désormais des cibles principales pour les attaques de la chaîne d’approvisionnement. 
-**Scénario #4 :** Les composants fonctionnent généralement avec les mêmes privilèges que l’application elle-même, donc des défauts dans n’importe quel composant peuvent avoir un impact sérieux. Ces défauts peuvent être accidentels (par exemple, une erreur de codage) ou intentionnels (par exemple, une porte dérobée dans un composant). Voici quelques exemples de vulnérabilités exploitables de composants découverts : 
-* CVE-2017-5638, une vulnérabilité d’exécution de code à distance Struts 2 qui permet l’exécution de code arbitraire sur le serveur, a été tenue responsable de violations importantes. 
-* CVE-2021-44228 (« Log4Shell »), une vulnérabilité zero-day d’exécution de code à distance Apache Log4j, a été tenue responsable de campagnes de ransomware, de cryptominage et d’autres attaques. 
-Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A03_2025-Software_Supply_Chain_Failures/</t>
   </si>
   <si>
     <t>## Tableau des scores
@@ -5803,29 +5656,6 @@
 Para obtener más información sobre las referencias y la lista de CWE asociadas: https://top10.owasp.org/2025/es/A05_2025-Injection/</t>
   </si>
   <si>
-    <t>## جدول امتیازدهی
-| تعداد CWEهای نگاشت‌شده | بیشترین نرخ بروز | میانگین نرخ بروز | بیشترین پوشش | میانگین پوشش | میانگین امتیاز بهره‌برداری | میانگین امتیاز تأثیر | تعداد کل رخدادها |
-|-----------------------|-----------------|-----------------|---------------|---------------|----------------------------|----------------------|----------------|
-| 37                    | 13.77%          | 3.08%           | 100.00%       | 42.93%        | 7.15                       | 4.32                 | 1,404,249      |
-## چگونه جلوگیری کنیم
-- از API امن استفاده کنید یا از ORMها بهره ببرید تا داده از دستورات جدا شود.  
-- اگر جداسازی ممکن نیست:
-  - اعتبارسنجی مثبت سمت سرور انجام دهید  
-  - برای کوئری‌های باقی‌مانده، کاراکترهای ویژه را با syntax مخصوص interpreter escape کنید  
-  - توجه داشته باشید که ساختار SQL مانند table/column name را نمی‌توان escape کرد  
-⚠️ هشدار: این تکنیک‌ها پیچیده هستند و در صورت تغییرات جزئی سیستم خطاپذیر می‌شوند.
-## نمونه سناریوهای حمله
-**سناریو #1:**
-```java
-String query = "SELECT * FROM accounts WHERE custID='" + request.getParameter("id") + "'";
-سناریو #2:
-Query HQLQuery = session.createQuery("FROM accounts WHERE custID='" + request.getParameter("id") + "'");
-در هر دو، مهاجم مقدار id را به ' UNION SLEEP(10);-- تغییر می‌دهد:
-http://example.com/app/accountView?id=' UNION SELECT SLEEP(10);--
-این باعث بازگرداندن همه رکوردها می‌شود. حملات خطرناک‌تر می‌توانند داده‌ها را تغییر دهند، حذف کنند یا stored procedure اجرا کنند.
-برای اطلاعات بیشتر درباره منابع و فهرست CWEهای نگاشت‌شده: https://top10.owasp.org/2025/fa/A05_2025-Injection/</t>
-  </si>
-  <si>
     <t>## Tabella dei punteggi.
 &lt;table&gt;
   &lt;tr&gt;
@@ -8648,6 +8478,177 @@
 **场景 #2：** 错误处理不当或数据库错误把完整系统错误暴露给用户，导致敏感数据泄露。攻击者持续制造错误，以利用敏感系统信息构造更好的 SQL 注入攻击。用户错误消息中的敏感数据成为侦察信息。
 **场景 #3：** 攻击者通过网络中断打断多步骤交易，可能导致金融交易状态损坏。假设交易顺序为：扣减用户账户、增加目标账户余额、记录交易。如果系统在中途出错时没有正确回滚整个交易（故障关闭），攻击者可能耗尽用户账户，或可能利用竞争条件多次向目标账户转账。
 有關參考資料及已對應 CWE 清單的更多資訊： https://top10.owasp.org/2025/zh-Hant/A10_2025-Mishandling_of_Exceptional_Conditions/</t>
+  </si>
+  <si>
+    <t>## جدول امتیازدهی
+| تعداد CWEهای نگاشت‌شده | بیشترین نرخ بروز | میانگین نرخ بروز | بیشترین پوشش | میانگین پوشش | میانگین امتیاز بهره‌برداری | میانگین امتیاز تأثیر | تعداد کل رخدادها |
+|-----------------------|-----------------|-----------------|---------------|---------------|----------------------------|----------------------|----------------|
+| 37                    | 13.77%          | 3.08%           | 100.00%       | 42.93%        | 7.15                       | 4.32                 | 1,404,249      |
+## چگونه جلوگیری کنیم
+- از API امن استفاده کنید یا از ORMها بهره ببرید تا داده از دستورات جدا شود.  
+- اگر جداسازی ممکن نیست:
+  - اعتبارسنجی مثبت سمت سرور انجام دهید  
+  - برای کوئری‌های باقی‌مانده، کاراکترهای ویژه را با syntax مخصوص interpreter escape کنید  
+  - توجه داشته باشید که ساختار SQL مانند table/column name را نمی‌توان escape کرد  
+⚠️ هشدار: این تکنیک‌ها پیچیده هستند و در صورت تغییرات جزئی سیستم خطاپذیر می‌شوند.
+## نمونه سناریوهای حمله
+**سناریو #1:**
+```java
+String query = "SELECT * FROM accounts WHERE custID='" + request.getParameter("id") + "'";
+```
+سناریو #2:
+Query HQLQuery = session.createQuery("FROM accounts WHERE custID='" + request.getParameter("id") + "'");
+در هر دو، مهاجم مقدار id را به ' UNION SLEEP(10);-- تغییر می‌دهد:
+http://example.com/app/accountView?id=' UNION SELECT SLEEP(10);--
+این باعث بازگرداندن همه رکوردها می‌شود. حملات خطرناک‌تر می‌توانند داده‌ها را تغییر دهند، حذف کنند یا stored procedure اجرا کنند.
+برای اطلاعات بیشتر درباره منابع و فهرست CWEهای نگاشت‌شده: https://top10.owasp.org/2025/fa/A05_2025-Injection/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;6
+   &lt;/td&gt;
+   &lt;td&gt;9,56 % 
+   &lt;/td&gt;
+   &lt;td&gt;5,72 % 
+   &lt;/td&gt;
+   &lt;td&gt;65,42 % 
+   &lt;/td&gt;
+   &lt;td&gt;27,47 % 
+   &lt;/td&gt;
+   &lt;td&gt;8.17
+   &lt;/td&gt;
+   &lt;td&gt;5.23
+   &lt;/td&gt;
+   &lt;td&gt;215 248
+   &lt;/td&gt;
+   &lt;td&gt;11
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+Il devrait y avoir un processus de gestion des correctifs pour : 
+* Générer et gérer centralisément la liste des documents logiciels (SBOM) de l’ensemble de votre logiciel. 
+* Suivre non seulement vos dépendances directes, mais aussi leurs dépendances (transitives), et ainsi de suite. 
+* Réduire la surface d’attaque en supprimant les dépendances inutilisées, les fonctionnalités, les composants, les fichiers et la documentation inutiles. 
+* Inventorier continuellement les versions des composants côté client et côté serveur (par exemple, frameworks, bibliothèques) et leurs dépendances à l’aide d’outils comme OWASP Dependency Track, OWASP Dependency Check, retire.js, etc. 
+* Surveillez en continu des sources telles que Common Vulnerability and Exposures (CVE), National Vulnerability Database (NVD) et [Open Source Vulnerabilities (OSV)](https://osv.dev/) pour les vulnérabilités des composants que vous utilisez. Utilisez l’analyse de composition logicielle, la chaîne d’approvisionnement logicielle ou des outils SBOM axés sur la sécurité pour automatiser le processus. Abonnez-vous aux alertes concernant les vulnérabilités de sécurité liées aux composants que vous utilisez. 
+* N’obtenir les composants que de sources officielles (fiables) via des liens sécurisés. Privilégier les paquets signés pour réduire le risque d’inclure un composant modifié et malveillant (voir [A08:2025 - Défaillances d’intégrité logicielle et des données](https://owasp.org/Top10/2025/A08_2025-Software_or_Data_Integrity_Failures/)). 
+* Choisissez délibérément la version d’une dépendance que vous utilisez et ne mettez à jour que lorsqu’il y a un besoin. 
+* Surveillez les bibliothèques et composants non maintenus ou qui ne créent pas de correctifs de sécurité pour les versions précédentes. Si le patch n’est pas possible, envisagez de migrer vers une alternative. Si cela n’est pas possible, envisagez de déployer un correctif virtuel pour surveiller, détecter ou protéger contre le problème découvert. 
+* Mettez régulièrement à jour votre CI/CD, IDE et tout autre outil de développement
+* Éviter de déployer des mises à jour simultanément sur tous les systèmes. Utiliser des déploiements par étapes ou des déploiements canari pour limiter l’exposition au cas où un fournisseur de confiance serait compromis. 
+Il devrait y avoir un processus de gestion des changements ou un système de suivi pour suivre les modifications sur :
+* Paramètres CI/CD (tous les outils de compilation et pipelines)
+* Dépôts de code
+* Zones de bac à sable
+* IDE développeurs
+* Outils SBOM et artefacts créés
+* Systèmes de journalisation et journaux
+* Intégrations tierces, telles que le SaaS
+* Dépôts d’artefacts
+* Registres de conteneurs
+Renforcez les systèmes suivants, ce qui inclut la mise en service de la MFA et la fermeture de l’IAM : 
+* Votre dépôt de code (ce qui inclut de ne pas vérifier les secrets, protéger les branches, sauvegarder)
+* Stations de travail développeurs (correctifs réguliers, MFA, surveillance, et plus encore)
+* Votre serveur de compilation &amp; CI/CD (séparation des fonctions, contrôle d’accès, compilations signées, secrets à portée d’environnement, journaux inviolables, plus encore)
+* Vos artefacts (assurez l’intégrité via la provenance, la signature et l’horodatage, promouvez les artefacts plutôt que les reconstruisez pour chaque environnement, assurez-vous que les builds restent immuables)
+* Infrastructure en tant que code (géré comme tout le code, y compris l’utilisation des PR et le contrôle de versions)
+Chaque organisation doit s’assurer d’un plan continu pour la surveillance, le tri et l’application des mises à jour ou modifications de configuration tout au long de la durée de vie de l’application ou du portefeuille.
+## Exemples de scénarios d’attaque
+**Scénario #1 :** Un fournisseur de confiance est compromis par des logiciels malveillants, ce qui entraîne la compromission de vos systèmes informatiques lors de la mise à jour. L’exemple le plus célèbre est probablement : 
+* Le compromis SolarWinds de 2019 qui a conduit à la compromission de ~18 000 organisations. [https://www.npr.org/2021/04/16/985439655/a-worst-nightmare-cyberattack-the-untold-story-of-the-solarwinds-hack](https://www.npr.org/2021/04/16/985439655/a-worst-nightmare-cyberattack-the-untold-story-of-the-solarwinds-hack)
+**Scénario #2 :** Un fournisseur de confiance est compromis au point de ne se comporter de manière malveillante que dans une condition spécifique. 
+* Le vol de 1,5 milliard de dollars par Bybit en 2025 a été causé par [une attaque de chaîne d’approvisionnement dans un logiciel de portefeuille](https://www.sygnia.co/blog/sygnia-investigation-bybit-hack/) qui ne s’est exécutée que lorsque le portefeuille cible était utilisé. 
+**Scénario #3 :** L’attaque de chaîne d’approvisionnement ['Shai-Hulud'](https://www.cisa.gov/news-events/alerts/2025/09/23/widespread-supply-chain-compromise-impacting-npm-ecosystem) en 2025 a été le premier ver npm auto-propagant réussi. Les attaques ont semé des versions malveillantes de paquets populaires, qui utilisaient un script post-installation pour récolter et exfiltrer des données sensibles vers des dépôts publics GitHub. Le malware détectait également les jetons npm dans l’environnement victime et les utilisait automatiquement pour diffuser des versions malveillantes de tout package accessible. Le ver a atteint plus de 500 versions de paquets avant d’être perturbé par npm. Cette attaque de chaîne d’approvisionnement était avancée, se propageait rapidement et causait des dommages, et en ciblant les machines développeurs, elle a démontré que les développeurs eux-mêmes sont désormais des cibles principales pour les attaques de la chaîne d’approvisionnement. 
+**Scénario #4 :** Les composants fonctionnent généralement avec les mêmes privilèges que l’application elle-même, donc des défauts dans n’importe quel composant peuvent avoir un impact sérieux. Ces défauts peuvent être accidentels (par exemple, une erreur de codage) ou intentionnels (par exemple, une porte dérobée dans un composant). Voici quelques exemples de vulnérabilités exploitables de composants découverts : 
+* CVE-2017-5638, une vulnérabilité d’exécution de code à distance Struts 2 qui permet l’exécution de code arbitraire sur le serveur, a été tenue responsable de violations importantes. 
+* CVE-2021-44228 (« Log4Shell »), une vulnérabilité zero-day d’exécution de code à distance Apache Log4j, a été tenue responsable de campagnes de ransomware, de cryptominage et d’autres attaques. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A03_2025-Software_Supply_Chain_Failures/</t>
+  </si>
+  <si>
+    <t>## Tableau des scores
+&lt;table&gt;
+  &lt;tr&gt;
+   &lt;td&gt;CWEs cartographiées 
+   &lt;/td&gt;
+   &lt;td&gt;Taux d’incidence maximal
+   &lt;/td&gt;
+   &lt;td&gt;Taux moyen d’incidence
+   &lt;/td&gt;
+   &lt;td&gt;Couverture maximale
+   &lt;/td&gt;
+   &lt;td&gt;Couverture moyenne
+   &lt;/td&gt;
+   &lt;td&gt;Exploit pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Impact pondéré moyen
+   &lt;/td&gt;
+   &lt;td&gt;Occurrences totales
+   &lt;/td&gt;
+   &lt;td&gt;Total des CVE
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td&gt;36
+   &lt;/td&gt;
+   &lt;td&gt;15,80 % 
+   &lt;/td&gt;
+   &lt;td&gt;2,92 % 
+   &lt;/td&gt;
+   &lt;td&gt;100,00 % 
+   &lt;/td&gt;
+   &lt;td&gt;37,14 % 
+   &lt;/td&gt;
+   &lt;td&gt;7,69
+   &lt;/td&gt;
+   &lt;td&gt;4,44
+   &lt;/td&gt;
+   &lt;td&gt;1 120 673
+   &lt;/td&gt;
+   &lt;td&gt;7 147
+   &lt;/td&gt;
+  &lt;/tr&gt;
+&lt;/table&gt;
+## Comment prévenir
+* Lorsque possible, implémenter et faire respecter l’utilisation de l’authentification multifactorielle pour prévenir le bourrage automatisé des identifiants, la force brute et les attaques de réutilisation de crédents volées. 
+* Lorsque possible, encourager et activer l’utilisation de gestionnaires de mots de passe pour aider les utilisateurs à faire de meilleurs choix. 
+* Ne pas livrer ni déployer avec des identifiants par défaut, en particulier pour les utilisateurs administrateurs. 
+* Mettre en place des vérifications de mots de passe faibles, comme tester de nouveaux mots de passe ou modifiés dans la liste des 10 000 pires mots de passe. 
+* Lors de la création d’un nouveau compte et des changements de mot de passe, validez contre les listes d’identifiants connus pour violation (par exemple : utiliser [haveibeenpwned.com](https://haveibeenpwned.com)). 
+* Aligner les politiques de longueur, de complexité et de rotation des mots de passe avec les directives du [National Institute of Standards and Technology (NIST) 800-63b dans la section 5.1.1](https://pages.nist.gov/800-63-3/sp800-63b.html#:~:text=5.1.1%20Memorized%20Secrets) pour les secrets mémorisés ou d’autres politiques modernes fondées sur des mots de passe fondées sur des preuves. 
+* Ne forcez pas les êtres humains à faire tourner les mots de passe sauf si vous suspectez une faille. Si vous soupçonnez une fuite, forcez immédiatement la réinitialisation du mot de passe.  
+* S’assurer que l’enregistrement, la récupération des identifiants et les voies API sont renforcés contre les attaques d’énumération de comptes en utilisant les mêmes messages pour tous les résultats (« Nom d’utilisateur ou mot de passe invalides. »). 
+* Limiter ou retarder de plus en plus les tentatives de connexion ratées, mais veillez à ne pas créer un scénario de déni de service. Consignez toutes les défaillances et alertez les administrateurs lorsque des attaques de type « credentialsal stuffing, de force brute » ou d’autres attaques sont détectées ou suspectées. 
+* Utiliser un gestionnaire de session intégré sécurisé côté serveur qui génère un nouvel ID de session aléatoire avec une forte entropie après la connexion. Les identifiants de session ne doivent pas être dans l’URL, être stockés de manière sécurisée dans un cookie sécurisé, et invalidés après déconnexion, inactivité et délais absolus.  
+* Idéalement, utiliser un système préfabriqué et bien fiable pour gérer l’authentification, l’identité et la gestion des sessions. Transférez ce risque autant que possible en achetant et en utilisant un système renforcé et bien testé. 
+* Vérifier l’utilisation prévue des identifiants fournis, par exemple pour les JWT, valider les affirmations « aud », « iss » et les périmètres
+## Exemples de scénarios d’attaque
+**Scénario #1 :** Le remplissage de crédentiaux, l’utilisation de listes de combinaisons de noms d’utilisateur et de mots de passe connus, est désormais une attaque très courante. Plus récemment, les attaquants ont été observés « incrémentant » ou ajustant autrement les mots de passe, en fonction du comportement humain courant. Par exemple, changer « Winter2025 » en « Hiver 2026 », ou « ILoveMyDog6 » en « ILoveMyDog7 » ou « ILoveMyDog5 ». Cet ajustement des tentatives de mot de passe est appelé attaque hybride de remplissage de crédibles ou attaque par pulvérisation de mots de passe, et ils peuvent être encore plus efficaces que la version traditionnelle. Si une application ne met pas en place de défenses contre les menaces automatisées (force brute, scripts ou bots) ou bourrage de crédents, l’application peut être utilisée comme oracle de mot de passe pour déterminer si les identifiants sont valides et obtenir un accès non autorisé. 
+**Scénario #2 :** La plupart des attaques d’authentification réussies surviennent en raison de l’utilisation continue des mots de passe comme seul facteur d’authentification. Une fois considérées comme les meilleures pratiques, la rotation des mots de passe et les exigences de complexité encouragent les utilisateurs à réutiliser les mots de passe et à utiliser des mots de passe faibles. Il est recommandé aux organisations d’arrêter ces pratiques conformément au NIST 800-63 et d’imposer l’utilisation de l’authentification multifacteur sur tous les systèmes importants. 
+**Scénario #3 :** Les délais d’expiration des sessions d’application ne sont pas correctement implémentés. Un utilisateur utilise un ordinateur public pour accéder à une application et au lieu de sélectionner « déconnexion », il ferme simplement l’onglet du navigateur et s’en va. Un autre exemple est si une session de connexion unique (SSO) ne peut pas être fermée par un seul déconnexion (SLO). C’est-à-dire qu’une seule connexion vous connecte, par exemple, à votre lecteur de messagerie, à votre système de documents et à votre système de chat. Mais la déconnexion ne se produit qu’au système actuel. Si un attaquant utilise le même navigateur après que la victime pense s’être déconnectée avec succès, mais avec l’utilisateur toujours authentifié sur certaines applications, il peut alors accéder au compte de la victime. Le même problème peut survenir dans les bureaux et les entreprises lorsqu’une application sensible n’a pas été correctement fermée et qu’un collègue a un accès (temporaire) à l’ordinateur déverrouillé. 
+Pour plus d’informations sur les références et la liste des CWE cartographiées : https://top10.owasp.org/2025/A07_2025-Authentication_Failures/</t>
   </si>
 </sst>
 </file>
@@ -10441,7 +10442,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -10639,7 +10640,7 @@
         <v>50</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -10694,7 +10695,7 @@
         <v>8</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>10</v>
@@ -10801,7 +10802,7 @@
         <v>62</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>63</v>
@@ -10828,7 +10829,7 @@
         <v>68</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>69</v>
@@ -10837,7 +10838,7 @@
         <v>70</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>71</v>
@@ -10846,7 +10847,7 @@
         <v>72</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="R2" s="5" t="s">
         <v>73</v>
@@ -10855,7 +10856,7 @@
         <v>74</v>
       </c>
       <c r="T2" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="U2" s="5" t="s">
         <v>63</v>
@@ -10864,7 +10865,7 @@
         <v>75</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="X2" s="5" t="s">
         <v>76</v>
@@ -10873,7 +10874,7 @@
         <v>77</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="AA2" s="5" t="s">
         <v>78</v>
@@ -10882,7 +10883,7 @@
         <v>79</v>
       </c>
       <c r="AC2" s="5" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="AD2" s="5" t="s">
         <v>80</v>
@@ -10891,7 +10892,7 @@
         <v>81</v>
       </c>
       <c r="AF2" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="AG2" s="5" t="s">
         <v>82</v>
@@ -10900,7 +10901,7 @@
         <v>83</v>
       </c>
       <c r="AI2" s="5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -10908,7 +10909,7 @@
         <v>84</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>85</v>
@@ -10917,7 +10918,7 @@
         <v>86</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>87</v>
@@ -10926,7 +10927,7 @@
         <v>259</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>88</v>
@@ -10935,16 +10936,16 @@
         <v>89</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="L3" s="8" t="s">
         <v>90</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="O3" s="8" t="s">
         <v>91</v>
@@ -10953,7 +10954,7 @@
         <v>92</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="R3" s="8" t="s">
         <v>93</v>
@@ -10962,7 +10963,7 @@
         <v>94</v>
       </c>
       <c r="T3" s="8" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="U3" s="8" t="s">
         <v>85</v>
@@ -10971,7 +10972,7 @@
         <v>95</v>
       </c>
       <c r="W3" s="8" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="X3" s="8" t="s">
         <v>96</v>
@@ -10980,7 +10981,7 @@
         <v>97</v>
       </c>
       <c r="Z3" s="8" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="AA3" s="8" t="s">
         <v>98</v>
@@ -10989,7 +10990,7 @@
         <v>99</v>
       </c>
       <c r="AC3" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="AD3" s="8" t="s">
         <v>100</v>
@@ -10998,7 +10999,7 @@
         <v>101</v>
       </c>
       <c r="AF3" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AG3" s="8" t="s">
         <v>102</v>
@@ -11007,7 +11008,7 @@
         <v>103</v>
       </c>
       <c r="AI3" s="8" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -11015,7 +11016,7 @@
         <v>104</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>105</v>
@@ -11027,13 +11028,13 @@
         <v>107</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>260</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>271</v>
+        <v>396</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>108</v>
@@ -11042,7 +11043,7 @@
         <v>109</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>110</v>
@@ -11051,7 +11052,7 @@
         <v>111</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="O4" s="5" t="s">
         <v>112</v>
@@ -11060,7 +11061,7 @@
         <v>113</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>114</v>
@@ -11069,7 +11070,7 @@
         <v>115</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="U4" s="5" t="s">
         <v>105</v>
@@ -11078,7 +11079,7 @@
         <v>116</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="X4" s="5" t="s">
         <v>117</v>
@@ -11087,7 +11088,7 @@
         <v>118</v>
       </c>
       <c r="Z4" s="5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="AA4" s="5" t="s">
         <v>105</v>
@@ -11105,7 +11106,7 @@
         <v>121</v>
       </c>
       <c r="AF4" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AG4" s="5" t="s">
         <v>122</v>
@@ -11114,7 +11115,7 @@
         <v>123</v>
       </c>
       <c r="AI4" s="5" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -11122,7 +11123,7 @@
         <v>124</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>125</v>
@@ -11149,7 +11150,7 @@
         <v>130</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>131</v>
@@ -11158,7 +11159,7 @@
         <v>132</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="O5" s="8" t="s">
         <v>133</v>
@@ -11167,7 +11168,7 @@
         <v>134</v>
       </c>
       <c r="Q5" s="8" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="R5" s="8" t="s">
         <v>135</v>
@@ -11176,7 +11177,7 @@
         <v>136</v>
       </c>
       <c r="T5" s="8" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U5" s="8" t="s">
         <v>125</v>
@@ -11185,7 +11186,7 @@
         <v>137</v>
       </c>
       <c r="W5" s="8" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="X5" s="8" t="s">
         <v>138</v>
@@ -11194,7 +11195,7 @@
         <v>139</v>
       </c>
       <c r="Z5" s="8" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="AA5" s="8" t="s">
         <v>140</v>
@@ -11203,7 +11204,7 @@
         <v>141</v>
       </c>
       <c r="AC5" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="AD5" s="8" t="s">
         <v>142</v>
@@ -11212,7 +11213,7 @@
         <v>143</v>
       </c>
       <c r="AF5" s="8" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="AG5" s="8" t="s">
         <v>144</v>
@@ -11221,7 +11222,7 @@
         <v>145</v>
       </c>
       <c r="AI5" s="8" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="6" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -11229,7 +11230,7 @@
         <v>146</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>147</v>
@@ -11256,7 +11257,7 @@
         <v>151</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>147</v>
@@ -11265,7 +11266,7 @@
         <v>152</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>153</v>
@@ -11274,7 +11275,7 @@
         <v>154</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>155</v>
@@ -11283,7 +11284,7 @@
         <v>156</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>347</v>
+        <v>395</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>147</v>
@@ -11292,7 +11293,7 @@
         <v>157</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="X6" s="5" t="s">
         <v>158</v>
@@ -11301,7 +11302,7 @@
         <v>159</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="AA6" s="5" t="s">
         <v>160</v>
@@ -11310,7 +11311,7 @@
         <v>161</v>
       </c>
       <c r="AC6" s="5" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="AD6" s="5" t="s">
         <v>162</v>
@@ -11319,7 +11320,7 @@
         <v>163</v>
       </c>
       <c r="AF6" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="AG6" s="5" t="s">
         <v>164</v>
@@ -11328,7 +11329,7 @@
         <v>165</v>
       </c>
       <c r="AI6" s="5" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="7" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -11336,7 +11337,7 @@
         <v>166</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>167</v>
@@ -11354,7 +11355,7 @@
         <v>265</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>171</v>
@@ -11363,7 +11364,7 @@
         <v>172</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="L7" s="8" t="s">
         <v>173</v>
@@ -11372,7 +11373,7 @@
         <v>174</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="O7" s="8" t="s">
         <v>175</v>
@@ -11381,7 +11382,7 @@
         <v>176</v>
       </c>
       <c r="Q7" s="8" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="R7" s="8" t="s">
         <v>167</v>
@@ -11390,7 +11391,7 @@
         <v>177</v>
       </c>
       <c r="T7" s="8" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="U7" s="8" t="s">
         <v>167</v>
@@ -11399,7 +11400,7 @@
         <v>178</v>
       </c>
       <c r="W7" s="8" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="X7" s="8" t="s">
         <v>179</v>
@@ -11408,7 +11409,7 @@
         <v>180</v>
       </c>
       <c r="Z7" s="8" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="AA7" s="8" t="s">
         <v>181</v>
@@ -11417,7 +11418,7 @@
         <v>182</v>
       </c>
       <c r="AC7" s="8" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="AD7" s="8" t="s">
         <v>183</v>
@@ -11426,7 +11427,7 @@
         <v>184</v>
       </c>
       <c r="AF7" s="8" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="AG7" s="8" t="s">
         <v>185</v>
@@ -11435,7 +11436,7 @@
         <v>186</v>
       </c>
       <c r="AI7" s="8" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="8" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -11443,7 +11444,7 @@
         <v>187</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>188</v>
@@ -11461,7 +11462,7 @@
         <v>263</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>269</v>
+        <v>397</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>192</v>
@@ -11470,7 +11471,7 @@
         <v>193</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>194</v>
@@ -11479,7 +11480,7 @@
         <v>195</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="O8" s="5" t="s">
         <v>196</v>
@@ -11488,7 +11489,7 @@
         <v>197</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="R8" s="5" t="s">
         <v>188</v>
@@ -11497,7 +11498,7 @@
         <v>198</v>
       </c>
       <c r="T8" s="5" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="U8" s="5" t="s">
         <v>188</v>
@@ -11506,16 +11507,16 @@
         <v>199</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="X8" s="5" t="s">
         <v>200</v>
       </c>
       <c r="Y8" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="Z8" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="AA8" s="5" t="s">
         <v>201</v>
@@ -11524,7 +11525,7 @@
         <v>202</v>
       </c>
       <c r="AC8" s="5" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="AD8" s="5" t="s">
         <v>203</v>
@@ -11533,7 +11534,7 @@
         <v>204</v>
       </c>
       <c r="AF8" s="5" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="AG8" s="5" t="s">
         <v>205</v>
@@ -11542,7 +11543,7 @@
         <v>206</v>
       </c>
       <c r="AI8" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="9" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -11550,7 +11551,7 @@
         <v>207</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>208</v>
@@ -11562,13 +11563,13 @@
         <v>210</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>264</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>211</v>
@@ -11577,7 +11578,7 @@
         <v>212</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="L9" s="8" t="s">
         <v>213</v>
@@ -11586,7 +11587,7 @@
         <v>214</v>
       </c>
       <c r="N9" s="8" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="O9" s="8" t="s">
         <v>215</v>
@@ -11595,7 +11596,7 @@
         <v>216</v>
       </c>
       <c r="Q9" s="8" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="R9" s="8" t="s">
         <v>208</v>
@@ -11604,7 +11605,7 @@
         <v>217</v>
       </c>
       <c r="T9" s="8" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="U9" s="8" t="s">
         <v>208</v>
@@ -11613,7 +11614,7 @@
         <v>218</v>
       </c>
       <c r="W9" s="8" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="X9" s="8" t="s">
         <v>219</v>
@@ -11622,7 +11623,7 @@
         <v>220</v>
       </c>
       <c r="Z9" s="8" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="AA9" s="8" t="s">
         <v>221</v>
@@ -11631,7 +11632,7 @@
         <v>222</v>
       </c>
       <c r="AC9" s="8" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="AD9" s="8" t="s">
         <v>223</v>
@@ -11640,7 +11641,7 @@
         <v>224</v>
       </c>
       <c r="AF9" s="8" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="AG9" s="8" t="s">
         <v>225</v>
@@ -11649,7 +11650,7 @@
         <v>226</v>
       </c>
       <c r="AI9" s="8" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
     </row>
     <row r="10" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -11657,52 +11658,52 @@
         <v>227</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>228</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>229</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>230</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>231</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="O10" s="5" t="s">
         <v>232</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="R10" s="5" t="s">
         <v>233</v>
@@ -11711,52 +11712,52 @@
         <v>234</v>
       </c>
       <c r="T10" s="5" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="U10" s="5" t="s">
         <v>228</v>
       </c>
       <c r="V10" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="X10" s="5" t="s">
         <v>235</v>
       </c>
       <c r="Y10" s="5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="Z10" s="5" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="AA10" s="5" t="s">
         <v>236</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="AC10" s="5" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="AD10" s="5" t="s">
         <v>237</v>
       </c>
       <c r="AE10" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="AF10" s="5" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="AG10" s="5" t="s">
         <v>238</v>
       </c>
       <c r="AH10" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="AI10" s="5" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="11" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -11764,25 +11765,25 @@
         <v>239</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>240</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>241</v>
@@ -11791,7 +11792,7 @@
         <v>242</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="L11" s="8" t="s">
         <v>243</v>
@@ -11800,7 +11801,7 @@
         <v>244</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="O11" s="8" t="s">
         <v>245</v>
@@ -11809,7 +11810,7 @@
         <v>246</v>
       </c>
       <c r="Q11" s="8" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="R11" s="8" t="s">
         <v>240</v>
@@ -11818,7 +11819,7 @@
         <v>247</v>
       </c>
       <c r="T11" s="8" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="U11" s="8" t="s">
         <v>240</v>
@@ -11827,7 +11828,7 @@
         <v>248</v>
       </c>
       <c r="W11" s="8" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="X11" s="8" t="s">
         <v>249</v>
@@ -11836,7 +11837,7 @@
         <v>250</v>
       </c>
       <c r="Z11" s="8" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="AA11" s="8" t="s">
         <v>251</v>
@@ -11845,7 +11846,7 @@
         <v>252</v>
       </c>
       <c r="AC11" s="8" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="AD11" s="8" t="s">
         <v>253</v>
@@ -11854,7 +11855,7 @@
         <v>254</v>
       </c>
       <c r="AF11" s="8" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="AG11" s="8" t="s">
         <v>255</v>
@@ -11863,7 +11864,7 @@
         <v>256</v>
       </c>
       <c r="AI11" s="8" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>